<commit_message>
Adversarial pass fixes across Rules, matrix, summary and models
Rules: Sec. 13.4 VAT reference covers logistics VAT (18(f)); Part 1
billing heading limited to the FCC; billing statement no longer uses
'Capacity Recovery Fee' (Sec. 28); short 'Superseded 19 Oct' notes on
12 older comments that still described the CLLC inside the GAT Price.

Matrix: capex rows 119, 411, 412, 441, 462 updated for the new-build
capex used in the models.

Summary: TOR_Conditions logistics note corrected; References lists the
new-build capex working assumption.

Models: Instructions no longer tell users to add logistics into F37;
sensitivity case label shows the current capex. GATP unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6VUATAmWPQdQ6XxJGJU7F
</commit_message>
<xml_diff>
--- a/FinModel_Summary.xlsx
+++ b/FinModel_Summary.xlsx
@@ -17237,70 +17237,70 @@
       </c>
       <c r="F155" s="123" t="inlineStr"/>
       <c r="G155" s="150" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="H155" s="150" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="J155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="N155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="P155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="R155" s="150" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="S155" s="150" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="T155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="U155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="V155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="W155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="X155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Y155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AB155" s="151" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="156" ht="15" customHeight="1">
@@ -18092,6 +18092,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -18374,10 +18375,11 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>How the TOR enters the models: capacity factor (Fin42 = 42%, top of band); Lot 1 non-mid-merit energy paid fuel only (TOR 4.2.2); grid (Visayas logistics caps); technology (TOR 2.6 lists CCGT, OCGT, reciprocating engines).</t>
+          <t>How the TOR enters the models: capacity factor (Fin42 = 42%, top of band); Lot 1 non-mid-merit energy paid fuel only (TOR 4.2.2); grid (Visayas logistics caps now affect only the Fuel Cost, not the GATP, after the 19 Oct 2026 decision); technology (TOR 2.6 lists CCGT, OCGT, reciprocating engines).</t>
         </is>
       </c>
     </row>
@@ -19187,7 +19189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -19440,6 +19442,23 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>New-build capital cost (working assumption, 20 Oct 2026): CCGT US$1,200/kW, gas engine US$1,100/kW, OCGT US$700/kW</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Market-level working values chosen 20 Oct 2026 in response to Wärtsilä and Quezon Power comments (GAIR matrix rows 119, 412); to be sourced in the Reference Parameters Resolution</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>models Fin42/Fin90, cell O34</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Raise capex to market +25% and re-solve all 22 models; add draft-rates deck
Existing CCGT US$600/kW; new CCGT 1,500, gas engine 1,375, OCGT 875.
FinModel_Summary, matrix capex remarks and the FGD deck updated. New
ERC_GATP_Rates_and_Assumptions.pptx opens with an executive summary of
draft GAT Prices by lot (Case A and B) before the assumption slides.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6VUATAmWPQdQ6XxJGJU7F
</commit_message>
<xml_diff>
--- a/FinModel_Summary.xlsx
+++ b/FinModel_Summary.xlsx
@@ -1646,7 +1646,7 @@
     <row r="2">
       <c r="A2" s="70" t="inlineStr">
         <is>
-          <t>Decision of 19 Oct 2026 (GAIR Sec. 8.6): GATP = CRF + OM; CLLC paid through the Fuel Cost. New-build capex: CCGT US$1,200/kW, gas engine US$1,100/kW, OCGT US$700/kW. PhP/kWh, excluding fuel.</t>
+          <t>Decision of 19 Oct 2026 (GAIR Sec. 8.6): GATP = CRF + OM; CLLC paid through the Fuel Cost. Capex (market +25%): existing CCGT US$600/kW; new CCGT US$1,500/kW, gas engine US$1,375/kW, OCGT US$875/kW. PhP/kWh, excluding fuel.</t>
         </is>
       </c>
       <c r="B2" s="69" t="n"/>
@@ -1698,28 +1698,28 @@
     <row r="5" ht="30" customHeight="1">
       <c r="B5" s="73" t="inlineStr">
         <is>
-          <t>1.09 – 1.72</t>
+          <t>1.35 – 2.12</t>
         </is>
       </c>
       <c r="C5" s="72" t="n"/>
       <c r="D5" s="72" t="n"/>
       <c r="F5" s="73" t="inlineStr">
         <is>
-          <t>2.61 – 3.84</t>
+          <t>3.18 – 4.70</t>
         </is>
       </c>
       <c r="G5" s="72" t="n"/>
       <c r="H5" s="72" t="n"/>
       <c r="J5" s="73" t="inlineStr">
         <is>
-          <t>1.73 – 2.44</t>
+          <t>2.06 – 2.92</t>
         </is>
       </c>
       <c r="K5" s="72" t="n"/>
       <c r="L5" s="72" t="n"/>
       <c r="N5" s="73" t="inlineStr">
         <is>
-          <t>2.54 – 3.68</t>
+          <t>3.05 – 4.45</t>
         </is>
       </c>
       <c r="O5" s="72" t="n"/>
@@ -1989,16 +1989,16 @@
         <v>0.42</v>
       </c>
       <c r="F6" s="82" t="n">
-        <v>1.113210815556326</v>
+        <v>1.486830198990387</v>
       </c>
       <c r="G6" s="82" t="n">
-        <v>0.04248573913293401</v>
+        <v>0.04777779558966159</v>
       </c>
       <c r="H6" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I6" s="82" t="n">
-        <v>0.1083414537470186</v>
+        <v>0.1328416046460465</v>
       </c>
       <c r="J6" s="83">
         <f>SUM(F6:I6)</f>
@@ -2008,7 +2008,7 @@
         <v>0.2408352664316716</v>
       </c>
       <c r="L6" s="84" t="n">
-        <v>0.2122220862959302</v>
+        <v>0.215260421728373</v>
       </c>
       <c r="M6" s="85">
         <f>K6+L6</f>
@@ -2025,7 +2025,7 @@
         <v>2.933449032397625</v>
       </c>
       <c r="Q6" s="89">
-        <f>IF(ABS(N6-1.7170953612)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N6-2.1235452874)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2052,16 +2052,16 @@
         <v>0.42</v>
       </c>
       <c r="F7" s="82" t="n">
-        <v>1.114523660438694</v>
+        <v>1.488143043872764</v>
       </c>
       <c r="G7" s="82" t="n">
-        <v>0.03800360248121382</v>
+        <v>0.04329565893794141</v>
       </c>
       <c r="H7" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I7" s="82" t="n">
-        <v>0.107633003568228</v>
+        <v>0.1321331544672561</v>
       </c>
       <c r="J7" s="83">
         <f>SUM(F7:I7)</f>
@@ -2071,7 +2071,7 @@
         <v>0.2408352664316718</v>
       </c>
       <c r="L7" s="84" t="n">
-        <v>0.1383289394592217</v>
+        <v>0.1413672748916645</v>
       </c>
       <c r="M7" s="85">
         <f>K7+L7</f>
@@ -2088,7 +2088,7 @@
         <v>2.413367717709602</v>
       </c>
       <c r="Q7" s="89">
-        <f>IF(ABS(N7-1.6393244724)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N7-2.0457743986)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2115,16 +2115,16 @@
         <v>0.42</v>
       </c>
       <c r="F8" s="82" t="n">
-        <v>3.153855737078547</v>
+        <v>3.94390173844531</v>
       </c>
       <c r="G8" s="82" t="n">
-        <v>0.06085164375219657</v>
+        <v>0.07052284750191348</v>
       </c>
       <c r="H8" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="82" t="n">
-        <v>0.2339831193583159</v>
+        <v>0.2839542902423469</v>
       </c>
       <c r="J8" s="83">
         <f>SUM(F8:I8)</f>
@@ -2134,7 +2134,7 @@
         <v>0.2408352664316718</v>
       </c>
       <c r="L8" s="84" t="n">
-        <v>0.1514475454490726</v>
+        <v>0.1570000865580744</v>
       </c>
       <c r="M8" s="85">
         <f>K8+L8</f>
@@ -2151,7 +2151,7 @@
         <v>3.729301496810136</v>
       </c>
       <c r="Q8" s="89">
-        <f>IF(ABS(N8-3.8409733121)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N8-4.6962142292)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2178,16 +2178,16 @@
         <v>0.42</v>
       </c>
       <c r="F9" s="82" t="n">
-        <v>1.784194928369909</v>
+        <v>2.23213977590294</v>
       </c>
       <c r="G9" s="82" t="n">
-        <v>0.04962773710894557</v>
+        <v>0.05544216248294227</v>
       </c>
       <c r="H9" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I9" s="82" t="n">
-        <v>0.1504877984741485</v>
+        <v>0.1794067985308676</v>
       </c>
       <c r="J9" s="83">
         <f>SUM(F9:I9)</f>
@@ -2197,7 +2197,7 @@
         <v>0.149314351908768</v>
       </c>
       <c r="L9" s="84" t="n">
-        <v>0.3041660054372468</v>
+        <v>0.3075042492329361</v>
       </c>
       <c r="M9" s="85">
         <f>K9+L9</f>
@@ -2214,7 +2214,7 @@
         <v>3.132474544268364</v>
       </c>
       <c r="Q9" s="89">
-        <f>IF(ABS(N9-2.4377908213)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N9-2.9238073381)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2241,16 +2241,16 @@
         <v>0.42</v>
       </c>
       <c r="F10" s="82" t="n">
-        <v>2.831870076237649</v>
+        <v>3.542161243792975</v>
       </c>
       <c r="G10" s="82" t="n">
-        <v>0.06917736992517988</v>
+        <v>0.07844986359632908</v>
       </c>
       <c r="H10" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I10" s="82" t="n">
-        <v>0.2174797461027427</v>
+        <v>0.2629041647027586</v>
       </c>
       <c r="J10" s="83">
         <f>SUM(F10:I10)</f>
@@ -2260,7 +2260,7 @@
         <v>0.2898455066464321</v>
       </c>
       <c r="L10" s="84" t="n">
-        <v>0.2668663304445173</v>
+        <v>0.2721899596042816</v>
       </c>
       <c r="M10" s="85">
         <f>K10+L10</f>
@@ -2277,7 +2277,7 @@
         <v>3.950128250112614</v>
       </c>
       <c r="Q10" s="89">
-        <f>IF(ABS(N10-3.6752390294)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N10-4.4455507383)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2304,16 +2304,16 @@
         <v>0.42</v>
       </c>
       <c r="F11" s="82" t="n">
-        <v>3.153836591657454</v>
+        <v>3.943882592731354</v>
       </c>
       <c r="G11" s="82" t="n">
-        <v>0.06080210844138251</v>
+        <v>0.07047331219180548</v>
       </c>
       <c r="H11" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="82" t="n">
-        <v>0.2340260628416754</v>
+        <v>0.2839972337237082</v>
       </c>
       <c r="J11" s="83">
         <f>SUM(F11:I11)</f>
@@ -2323,7 +2323,7 @@
         <v>0.2408352664316717</v>
       </c>
       <c r="L11" s="84" t="n">
-        <v>0.1514180498478056</v>
+        <v>0.1569705909572128</v>
       </c>
       <c r="M11" s="85">
         <f>K11+L11</f>
@@ -2340,7 +2340,7 @@
         <v>4.218436463045343</v>
       </c>
       <c r="Q11" s="89">
-        <f>IF(ABS(N11-3.8409180792)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N11-4.6961589960)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2367,16 +2367,16 @@
         <v>0.42</v>
       </c>
       <c r="F12" s="82" t="n">
-        <v>1.784178234915861</v>
+        <v>2.232123082103706</v>
       </c>
       <c r="G12" s="82" t="n">
-        <v>0.04957810000815011</v>
+        <v>0.05539252538226503</v>
       </c>
       <c r="H12" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I12" s="82" t="n">
-        <v>0.1505308275318445</v>
+        <v>0.1794498275846172</v>
       </c>
       <c r="J12" s="83">
         <f>SUM(F12:I12)</f>
@@ -2386,7 +2386,7 @@
         <v>0.149314351908768</v>
       </c>
       <c r="L12" s="84" t="n">
-        <v>0.304136451395162</v>
+        <v>0.3074746951909192</v>
       </c>
       <c r="M12" s="85">
         <f>K12+L12</f>
@@ -2403,7 +2403,7 @@
         <v>3.9183338116066</v>
       </c>
       <c r="Q12" s="89">
-        <f>IF(ABS(N12-2.4377379658)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N12-2.9237544822)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2430,16 +2430,16 @@
         <v>0.42</v>
       </c>
       <c r="F13" s="82" t="n">
-        <v>2.831854894884217</v>
+        <v>3.542146062279643</v>
       </c>
       <c r="G13" s="82" t="n">
-        <v>0.06912768448910267</v>
+        <v>0.07840017816032213</v>
       </c>
       <c r="H13" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I13" s="82" t="n">
-        <v>0.2175228191925891</v>
+        <v>0.2629472377908854</v>
       </c>
       <c r="J13" s="83">
         <f>SUM(F13:I13)</f>
@@ -2449,7 +2449,7 @@
         <v>0.2898455066464321</v>
       </c>
       <c r="L13" s="84" t="n">
-        <v>0.2668367486516327</v>
+        <v>0.2721603778114374</v>
       </c>
       <c r="M13" s="85">
         <f>K13+L13</f>
@@ -2466,7 +2466,7 @@
         <v>4.591637790993857</v>
       </c>
       <c r="Q13" s="89">
-        <f>IF(ABS(N13-3.6751876539)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N13-4.4454993627)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2493,16 +2493,16 @@
         <v>0.42</v>
       </c>
       <c r="F14" s="82" t="n">
-        <v>3.153840694143365</v>
+        <v>3.94388669530116</v>
       </c>
       <c r="G14" s="82" t="n">
-        <v>0.06081272315097044</v>
+        <v>0.07048392690121993</v>
       </c>
       <c r="H14" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I14" s="82" t="n">
-        <v>0.2340168606654816</v>
+        <v>0.2839880315481977</v>
       </c>
       <c r="J14" s="83">
         <f>SUM(F14:I14)</f>
@@ -2512,7 +2512,7 @@
         <v>0.2408352664316718</v>
       </c>
       <c r="L14" s="84" t="n">
-        <v>0.1514243703338647</v>
+        <v>0.1569769114431724</v>
       </c>
       <c r="M14" s="85">
         <f>K14+L14</f>
@@ -2529,7 +2529,7 @@
         <v>4.218448298406374</v>
       </c>
       <c r="Q14" s="89">
-        <f>IF(ABS(N14-3.8409299147)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N14-4.6961708316)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2556,16 +2556,16 @@
         <v>0.42</v>
       </c>
       <c r="F15" s="82" t="n">
-        <v>1.784181811973243</v>
+        <v>2.232126659257657</v>
       </c>
       <c r="G15" s="82" t="n">
-        <v>0.04958873652980943</v>
+        <v>0.05540316190389129</v>
       </c>
       <c r="H15" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="82" t="n">
-        <v>0.1505216070182965</v>
+        <v>0.1794406070721735</v>
       </c>
       <c r="J15" s="83">
         <f>SUM(F15:I15)</f>
@@ -2575,7 +2575,7 @@
         <v>0.149314351908768</v>
       </c>
       <c r="L15" s="84" t="n">
-        <v>0.3041427844042148</v>
+        <v>0.307481028199953</v>
       </c>
       <c r="M15" s="85">
         <f>K15+L15</f>
@@ -2592,7 +2592,7 @@
         <v>3.918345137513774</v>
       </c>
       <c r="Q15" s="89">
-        <f>IF(ABS(N15-2.4377492918)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N15-2.9237658083)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2619,16 +2619,16 @@
         <v>0.42</v>
       </c>
       <c r="F16" s="82" t="n">
-        <v>2.831858147979329</v>
+        <v>3.54214931541949</v>
       </c>
       <c r="G16" s="82" t="n">
-        <v>0.06913833136828895</v>
+        <v>0.07841082503948879</v>
       </c>
       <c r="H16" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I16" s="82" t="n">
-        <v>0.2175135892442209</v>
+        <v>0.2629380078429988</v>
       </c>
       <c r="J16" s="83">
         <f>SUM(F16:I16)</f>
@@ -2638,7 +2638,7 @@
         <v>0.2898455066464321</v>
       </c>
       <c r="L16" s="84" t="n">
-        <v>0.2668430876072663</v>
+        <v>0.2721667167670597</v>
       </c>
       <c r="M16" s="85">
         <f>K16+L16</f>
@@ -2655,7 +2655,7 @@
         <v>4.591648799911785</v>
       </c>
       <c r="Q16" s="89">
-        <f>IF(ABS(N16-3.6751986628)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N16-4.4455103717)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2776,16 +2776,16 @@
         <v>0.6680044139645122</v>
       </c>
       <c r="F20" s="82" t="n">
-        <v>0.700014289580048</v>
+        <v>0.9349231281474634</v>
       </c>
       <c r="G20" s="82" t="n">
-        <v>0.02680534643415587</v>
+        <v>0.03013266533409306</v>
       </c>
       <c r="H20" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I20" s="82" t="n">
-        <v>0.07938208693776358</v>
+        <v>0.09478627164445091</v>
       </c>
       <c r="J20" s="83">
         <f>SUM(F20:I20)</f>
@@ -2795,7 +2795,7 @@
         <v>0.1514223705513954</v>
       </c>
       <c r="L20" s="84" t="n">
-        <v>0.1349810410827771</v>
+        <v>0.1368913591210255</v>
       </c>
       <c r="M20" s="85">
         <f>K20+L20</f>
@@ -2812,7 +2812,7 @@
         <v>1.866648379916711</v>
       </c>
       <c r="Q20" s="89">
-        <f>IF(ABS(N20-1.0926051346)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N20-1.3481557948)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2839,16 +2839,16 @@
         <v>0.6680044139645122</v>
       </c>
       <c r="F21" s="82" t="n">
-        <v>0.700005694569188</v>
+        <v>0.9349145331365989</v>
       </c>
       <c r="G21" s="82" t="n">
-        <v>0.02677369187463278</v>
+        <v>0.03010101077456997</v>
       </c>
       <c r="H21" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I21" s="82" t="n">
-        <v>0.07940951372560666</v>
+        <v>0.09481369843229404</v>
       </c>
       <c r="J21" s="83">
         <f>SUM(F21:I21)</f>
@@ -2858,7 +2858,7 @@
         <v>0.1514223705513955</v>
       </c>
       <c r="L21" s="84" t="n">
-        <v>0.1349621965953671</v>
+        <v>0.1368725146336156</v>
       </c>
       <c r="M21" s="85">
         <f>K21+L21</f>
@@ -2875,7 +2875,7 @@
         <v>1.866616712646755</v>
       </c>
       <c r="Q21" s="89">
-        <f>IF(ABS(N21-1.0925734673)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N21-1.3481241275)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2902,16 +2902,16 @@
         <v>0.6312409193029385</v>
       </c>
       <c r="F22" s="82" t="n">
-        <v>2.097771885348189</v>
+        <v>2.623433816359344</v>
       </c>
       <c r="G22" s="82" t="n">
-        <v>0.04308338807996767</v>
+        <v>0.04951818254697807</v>
       </c>
       <c r="H22" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I22" s="82" t="n">
-        <v>0.1662610335270309</v>
+        <v>0.199509657197482</v>
       </c>
       <c r="J22" s="83">
         <f>SUM(F22:I22)</f>
@@ -2921,7 +2921,7 @@
         <v>0.1602412150546261</v>
       </c>
       <c r="L22" s="84" t="n">
-        <v>0.1440228049458968</v>
+        <v>0.1477172220764529</v>
       </c>
       <c r="M22" s="85">
         <f>K22+L22</f>
@@ -2938,7 +2938,7 @@
         <v>2.785909662514258</v>
       </c>
       <c r="Q22" s="89">
-        <f>IF(ABS(N22-2.6113803270)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N22-3.1804200932)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2965,16 +2965,16 @@
         <v>0.6312409193029385</v>
       </c>
       <c r="F23" s="82" t="n">
-        <v>1.185488649618506</v>
+        <v>1.483531489065016</v>
       </c>
       <c r="G23" s="82" t="n">
-        <v>0.03885971245045097</v>
+        <v>0.04272837587578042</v>
       </c>
       <c r="H23" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I23" s="82" t="n">
-        <v>0.1112574539563226</v>
+        <v>0.1304988872227758</v>
       </c>
       <c r="J23" s="83">
         <f>SUM(F23:I23)</f>
@@ -2984,7 +2984,7 @@
         <v>0.0993472157523211</v>
       </c>
       <c r="L23" s="84" t="n">
-        <v>0.299705284602134</v>
+        <v>0.3019264054948317</v>
       </c>
       <c r="M23" s="85">
         <f>K23+L23</f>
@@ -3001,7 +3001,7 @@
         <v>2.596631426479127</v>
       </c>
       <c r="Q23" s="89">
-        <f>IF(ABS(N23-1.7346583164)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N23-2.0580323734)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -3028,16 +3028,16 @@
         <v>0.6312409193029385</v>
       </c>
       <c r="F24" s="82" t="n">
-        <v>1.882837601322518</v>
+        <v>2.355434166676148</v>
       </c>
       <c r="G24" s="82" t="n">
-        <v>0.05095879864154527</v>
+        <v>0.05712830892326653</v>
       </c>
       <c r="H24" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I24" s="82" t="n">
-        <v>0.1556768036022249</v>
+        <v>0.185900217878147</v>
       </c>
       <c r="J24" s="83">
         <f>SUM(F24:I24)</f>
@@ -3047,7 +3047,7 @@
         <v>0.1928504776368586</v>
       </c>
       <c r="L24" s="84" t="n">
-        <v>0.259748028548601</v>
+        <v>0.2632901377160011</v>
       </c>
       <c r="M24" s="85">
         <f>K24+L24</f>
@@ -3064,7 +3064,7 @@
         <v>3.051306484962811</v>
       </c>
       <c r="Q24" s="89">
-        <f>IF(ABS(N24-2.5420717098)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N24-3.0546033088)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -3091,16 +3091,16 @@
         <v>0.6312409193029385</v>
       </c>
       <c r="F25" s="82" t="n">
-        <v>2.097759146825363</v>
+        <v>2.62342107764166</v>
       </c>
       <c r="G25" s="82" t="n">
-        <v>0.04305042945845613</v>
+        <v>0.04948522392593631</v>
       </c>
       <c r="H25" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I25" s="82" t="n">
-        <v>0.166289606235896</v>
+        <v>0.1995382299050175</v>
       </c>
       <c r="J25" s="83">
         <f>SUM(F25:I25)</f>
@@ -3110,7 +3110,7 @@
         <v>0.1602412150546261</v>
       </c>
       <c r="L25" s="84" t="n">
-        <v>0.1440031798674944</v>
+        <v>0.1476975969983202</v>
       </c>
       <c r="M25" s="85">
         <f>K25+L25</f>
@@ -3127,7 +3127,7 @@
         <v>3.275063111910242</v>
       </c>
       <c r="Q25" s="89">
-        <f>IF(ABS(N25-2.6113435774)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N25-3.1803833435)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -3154,16 +3154,16 @@
         <v>0.6312409193029385</v>
       </c>
       <c r="F26" s="82" t="n">
-        <v>1.185477542526925</v>
+        <v>1.483520381743764</v>
       </c>
       <c r="G26" s="82" t="n">
-        <v>0.03882668610235376</v>
+        <v>0.04269534952776186</v>
       </c>
       <c r="H26" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I26" s="82" t="n">
-        <v>0.1112860836025951</v>
+        <v>0.1305275168664224</v>
       </c>
       <c r="J26" s="83">
         <f>SUM(F26:I26)</f>
@@ -3173,7 +3173,7 @@
         <v>0.0993472157523211</v>
       </c>
       <c r="L26" s="84" t="n">
-        <v>0.2996856206397765</v>
+        <v>0.3019067415325195</v>
       </c>
       <c r="M26" s="85">
         <f>K26+L26</f>
@@ -3190,7 +3190,7 @@
         <v>3.382508381400652</v>
       </c>
       <c r="Q26" s="89">
-        <f>IF(ABS(N26-1.7346231486)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N26-2.0579972054)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -3217,16 +3217,16 @@
         <v>0.6312409193029385</v>
       </c>
       <c r="F27" s="82" t="n">
-        <v>1.882827500316316</v>
+        <v>2.355424065563553</v>
       </c>
       <c r="G27" s="82" t="n">
-        <v>0.05092574013327326</v>
+        <v>0.05709525041504129</v>
       </c>
       <c r="H27" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I27" s="82" t="n">
-        <v>0.1557054625455575</v>
+        <v>0.1859288768203355</v>
       </c>
       <c r="J27" s="83">
         <f>SUM(F27:I27)</f>
@@ -3236,7 +3236,7 @@
         <v>0.1928504776368586</v>
       </c>
       <c r="L27" s="84" t="n">
-        <v>0.2597283461220796</v>
+        <v>0.2632704552895065</v>
       </c>
       <c r="M27" s="85">
         <f>K27+L27</f>
@@ -3253,7 +3253,7 @@
         <v>3.692833237740226</v>
       </c>
       <c r="Q27" s="89">
-        <f>IF(ABS(N27-2.5420375268)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N27-3.0545691257)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -3280,16 +3280,16 @@
         <v>0.6312409193029385</v>
       </c>
       <c r="F28" s="82" t="n">
-        <v>2.097761876439413</v>
+        <v>2.623423807311532</v>
       </c>
       <c r="G28" s="82" t="n">
-        <v>0.04305749202029362</v>
+        <v>0.04949228648765837</v>
       </c>
       <c r="H28" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I28" s="82" t="n">
-        <v>0.1662834835117771</v>
+        <v>0.1995321071813534</v>
       </c>
       <c r="J28" s="83">
         <f>SUM(F28:I28)</f>
@@ -3299,7 +3299,7 @@
         <v>0.1602412150546261</v>
       </c>
       <c r="L28" s="84" t="n">
-        <v>0.1440073852414866</v>
+        <v>0.1477018023722461</v>
       </c>
       <c r="M28" s="85">
         <f>K28+L28</f>
@@ -3316,7 +3316,7 @@
         <v>3.275070986639969</v>
       </c>
       <c r="Q28" s="89">
-        <f>IF(ABS(N28-2.6113514523)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N28-3.1803912184)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -3343,16 +3343,16 @@
         <v>0.6312409193029385</v>
       </c>
       <c r="F29" s="82" t="n">
-        <v>1.185479922543897</v>
+        <v>1.483522761824987</v>
       </c>
       <c r="G29" s="82" t="n">
-        <v>0.03883376317698627</v>
+        <v>0.04270242660237237</v>
       </c>
       <c r="H29" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I29" s="82" t="n">
-        <v>0.1112799486776057</v>
+        <v>0.1305213819421677</v>
       </c>
       <c r="J29" s="83">
         <f>SUM(F29:I29)</f>
@@ -3362,7 +3362,7 @@
         <v>0.0993472157523211</v>
       </c>
       <c r="L29" s="84" t="n">
-        <v>0.299689834346019</v>
+        <v>0.3019109552387494</v>
       </c>
       <c r="M29" s="85">
         <f>K29+L29</f>
@@ -3379,7 +3379,7 @@
         <v>3.382515917162146</v>
       </c>
       <c r="Q29" s="89">
-        <f>IF(ABS(N29-1.7346306845)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N29-2.0580047414)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -3406,16 +3406,16 @@
         <v>0.6312409193029385</v>
       </c>
       <c r="F30" s="82" t="n">
-        <v>1.882829664783011</v>
+        <v>2.355426230060016</v>
       </c>
       <c r="G30" s="82" t="n">
-        <v>0.05093282409934952</v>
+        <v>0.05710233438110449</v>
       </c>
       <c r="H30" s="82" t="n">
         <v>0</v>
       </c>
       <c r="I30" s="82" t="n">
-        <v>0.1556993213430528</v>
+        <v>0.1859227356181512</v>
       </c>
       <c r="J30" s="83">
         <f>SUM(F30:I30)</f>
@@ -3425,7 +3425,7 @@
         <v>0.1928504776368586</v>
       </c>
       <c r="L30" s="84" t="n">
-        <v>0.2597325637849158</v>
+        <v>0.2632746729523353</v>
       </c>
       <c r="M30" s="85">
         <f>K30+L30</f>
@@ -3442,7 +3442,7 @@
         <v>3.692840562983414</v>
       </c>
       <c r="Q30" s="89">
-        <f>IF(ABS(N30-2.5420448516)&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(ABS(N30-3.0545764506)&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
     <row r="2">
       <c r="A2" s="70" t="inlineStr">
         <is>
-          <t>GATP = CRF + OM (decision of 19 Oct 2026); new-build capex at market levels. Previous-draft values kept for comparison.</t>
+          <t>GATP = CRF + OM (decision of 19 Oct 2026); capex at market +25%. Previous-draft values kept for comparison.</t>
         </is>
       </c>
       <c r="B2" s="69" t="n"/>
@@ -4098,10 +4098,10 @@
         <v>30</v>
       </c>
       <c r="F5" s="100" t="n">
-        <v>1.71709536116388</v>
+        <v>2.12354528738614</v>
       </c>
       <c r="G5" s="100" t="n">
-        <v>1.09260513458614</v>
+        <v>1.348155794798428</v>
       </c>
       <c r="H5" s="101">
         <f>G5-F5</f>
@@ -4137,10 +4137,10 @@
         <v>30</v>
       </c>
       <c r="F6" s="100" t="n">
-        <v>1.63932447237903</v>
+        <v>2.045774398601298</v>
       </c>
       <c r="G6" s="100" t="n">
-        <v>1.09257346731619</v>
+        <v>1.348124127528474</v>
       </c>
       <c r="H6" s="101">
         <f>G6-F6</f>
@@ -4176,10 +4176,10 @@
         <v>30</v>
       </c>
       <c r="F7" s="100" t="n">
-        <v>3.840973312069803</v>
+        <v>4.696214229179318</v>
       </c>
       <c r="G7" s="100" t="n">
-        <v>2.611380326955709</v>
+        <v>3.180420093234884</v>
       </c>
       <c r="H7" s="101">
         <f>G7-F7</f>
@@ -4215,10 +4215,10 @@
         <v>30</v>
       </c>
       <c r="F8" s="100" t="n">
-        <v>2.437790821299018</v>
+        <v>2.923807338058453</v>
       </c>
       <c r="G8" s="100" t="n">
-        <v>1.734658316379735</v>
+        <v>2.058032373410724</v>
       </c>
       <c r="H8" s="101">
         <f>G8-F8</f>
@@ -4254,10 +4254,10 @@
         <v>30</v>
       </c>
       <c r="F9" s="100" t="n">
-        <v>3.67523902935652</v>
+        <v>4.445550738342776</v>
       </c>
       <c r="G9" s="100" t="n">
-        <v>2.542071709751747</v>
+        <v>3.054603308830421</v>
       </c>
       <c r="H9" s="101">
         <f>G9-F9</f>
@@ -4293,10 +4293,10 @@
         <v>30</v>
       </c>
       <c r="F10" s="100" t="n">
-        <v>3.84091807921999</v>
+        <v>4.696158996035751</v>
       </c>
       <c r="G10" s="100" t="n">
-        <v>2.611343577441835</v>
+        <v>3.18038334352556</v>
       </c>
       <c r="H10" s="101">
         <f>G10-F10</f>
@@ -4332,10 +4332,10 @@
         <v>30</v>
       </c>
       <c r="F11" s="100" t="n">
-        <v>2.437737965759786</v>
+        <v>2.923754482170276</v>
       </c>
       <c r="G11" s="100" t="n">
-        <v>1.734623148623972</v>
+        <v>2.057997205422789</v>
       </c>
       <c r="H11" s="101">
         <f>G11-F11</f>
@@ -4371,10 +4371,10 @@
         <v>30</v>
       </c>
       <c r="F12" s="100" t="n">
-        <v>3.675187653863974</v>
+        <v>4.44549936268872</v>
       </c>
       <c r="G12" s="100" t="n">
-        <v>2.542037526754084</v>
+        <v>3.054569125725295</v>
       </c>
       <c r="H12" s="101">
         <f>G12-F12</f>
@@ -4410,10 +4410,10 @@
         <v>30</v>
       </c>
       <c r="F13" s="100" t="n">
-        <v>3.840929914725353</v>
+        <v>4.696170831625423</v>
       </c>
       <c r="G13" s="100" t="n">
-        <v>2.611351452267597</v>
+        <v>3.180391218407416</v>
       </c>
       <c r="H13" s="101">
         <f>G13-F13</f>
@@ -4449,10 +4449,10 @@
         <v>30</v>
       </c>
       <c r="F14" s="100" t="n">
-        <v>2.437749291834332</v>
+        <v>2.923765808342443</v>
       </c>
       <c r="G14" s="100" t="n">
-        <v>1.734630684496829</v>
+        <v>2.058004741360597</v>
       </c>
       <c r="H14" s="101">
         <f>G14-F14</f>
@@ -4488,10 +4488,10 @@
         <v>30</v>
       </c>
       <c r="F15" s="100" t="n">
-        <v>3.675198662845537</v>
+        <v>4.44551037171547</v>
       </c>
       <c r="G15" s="100" t="n">
-        <v>2.542044851647188</v>
+        <v>3.054576450648465</v>
       </c>
       <c r="H15" s="101">
         <f>G15-F15</f>
@@ -4559,7 +4559,7 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="106" t="inlineStr">
         <is>
-          <t>• New-build capital cost raised to current market levels (20 Oct 2026): CCGT US$1,200/kW (was 900), gas engine US$1,100/kW (was 850), OCGT US$700/kW (was 520). Equipment cost (F15) recalibrated and the GATP re-solved; existing Lots 1 and 2 unchanged.</t>
+          <t>• Capital cost raised to market +25% (20 Oct 2026): existing CCGT US$600/kW (was 450); new CCGT US$1,500/kW (was 1,200, originally 900), gas engine US$1,375/kW (1,100; 850), OCGT US$875/kW (700; 520). Equipment cost (F15) recalibrated and the GATP re-solved for all 22 models.</t>
         </is>
       </c>
     </row>
@@ -4735,7 +4735,7 @@
     <row r="2">
       <c r="A2" s="70" t="inlineStr">
         <is>
-          <t>Read from each model after the 20 Oct 2026 re-solve (CLLC out of the GATP; new-build capex CCGT US$1,200/kW, gas engine US$1,100/kW, OCGT US$700/kW). Values identical across Fin42 and Fin90 except capacity factor and results.</t>
+          <t>Read from each model after the 20 Oct 2026 re-solve (CLLC out of the GATP; capex at market +25%: existing CCGT US$600/kW, new CCGT US$1,500/kW, gas engine US$1,375/kW, OCGT US$875/kW). Values identical across Fin42 and Fin90 except capacity factor and results.</t>
         </is>
       </c>
       <c r="B2" s="69" t="n"/>
@@ -7057,74 +7057,74 @@
       </c>
       <c r="F35" s="123" t="inlineStr">
         <is>
-          <t>New-build raised 20 Oct 2026 to market levels: CCGT US$1,200/kW, gas engine US$1,100/kW, OCGT US$700/kW (were 900/850/520). Existing plants unchanged (brownfield US$450/kW).</t>
+          <t>Raised 20 Oct 2026 to market +25%: existing CCGT US$600/kW (was 450); new CCGT US$1,500/kW, gas engine US$1,375/kW, OCGT US$875/kW (were 1,200/1,100/700; originally 900/850/520).</t>
         </is>
       </c>
       <c r="G35" s="130" t="n">
-        <v>450</v>
+        <v>600</v>
       </c>
       <c r="H35" s="130" t="n">
-        <v>450</v>
+        <v>600</v>
       </c>
       <c r="I35" s="132" t="n">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="J35" s="132" t="n">
-        <v>700</v>
+        <v>875</v>
       </c>
       <c r="K35" s="132" t="n">
-        <v>1100</v>
+        <v>1375</v>
       </c>
       <c r="L35" s="132" t="n">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="M35" s="132" t="n">
-        <v>700</v>
+        <v>875</v>
       </c>
       <c r="N35" s="132" t="n">
-        <v>1100</v>
+        <v>1375</v>
       </c>
       <c r="O35" s="132" t="n">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="P35" s="132" t="n">
-        <v>700</v>
+        <v>875</v>
       </c>
       <c r="Q35" s="132" t="n">
-        <v>1100</v>
+        <v>1375</v>
       </c>
       <c r="R35" s="130" t="n">
-        <v>450</v>
+        <v>600</v>
       </c>
       <c r="S35" s="130" t="n">
-        <v>450</v>
+        <v>600</v>
       </c>
       <c r="T35" s="132" t="n">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="U35" s="132" t="n">
-        <v>700</v>
+        <v>875</v>
       </c>
       <c r="V35" s="132" t="n">
-        <v>1100</v>
+        <v>1375</v>
       </c>
       <c r="W35" s="132" t="n">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="X35" s="132" t="n">
-        <v>700</v>
+        <v>875</v>
       </c>
       <c r="Y35" s="132" t="n">
-        <v>1100</v>
+        <v>1375</v>
       </c>
       <c r="Z35" s="132" t="n">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="AA35" s="132" t="n">
-        <v>700</v>
+        <v>875</v>
       </c>
       <c r="AB35" s="132" t="n">
-        <v>1100</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="36" ht="24" customHeight="1">
@@ -7159,70 +7159,70 @@
         </is>
       </c>
       <c r="G36" s="133" t="n">
-        <v>450.0000000000019</v>
+        <v>599.9999999999998</v>
       </c>
       <c r="H36" s="133" t="n">
-        <v>450.0000000000015</v>
+        <v>599.9999999999999</v>
       </c>
       <c r="I36" s="134" t="n">
-        <v>1200.000000002668</v>
+        <v>1500.000000001293</v>
       </c>
       <c r="J36" s="134" t="n">
-        <v>700.0000000013767</v>
+        <v>875.000000000624</v>
       </c>
       <c r="K36" s="134" t="n">
-        <v>1100.000000000433</v>
+        <v>1375.000000000261</v>
       </c>
       <c r="L36" s="134" t="n">
-        <v>1200</v>
+        <v>1500.000000006675</v>
       </c>
       <c r="M36" s="134" t="n">
-        <v>700.0000000071039</v>
+        <v>875.0000000032207</v>
       </c>
       <c r="N36" s="134" t="n">
-        <v>1100.000000002231</v>
+        <v>1375.000000001347</v>
       </c>
       <c r="O36" s="134" t="n">
-        <v>1200</v>
+        <v>1500.000000005169</v>
       </c>
       <c r="P36" s="134" t="n">
-        <v>700.0000000055021</v>
+        <v>875.0000000024945</v>
       </c>
       <c r="Q36" s="134" t="n">
-        <v>1100.000000001727</v>
+        <v>1375.000000001044</v>
       </c>
       <c r="R36" s="133" t="n">
-        <v>450.0000000000019</v>
+        <v>599.9999999999998</v>
       </c>
       <c r="S36" s="133" t="n">
-        <v>450.0000000000015</v>
+        <v>599.9999999999999</v>
       </c>
       <c r="T36" s="134" t="n">
-        <v>1200.000000002668</v>
+        <v>1500.000000001293</v>
       </c>
       <c r="U36" s="134" t="n">
-        <v>700.0000000013767</v>
+        <v>875.000000000624</v>
       </c>
       <c r="V36" s="134" t="n">
-        <v>1100.000000000433</v>
+        <v>1375.000000000261</v>
       </c>
       <c r="W36" s="134" t="n">
-        <v>1200</v>
+        <v>1500.000000006675</v>
       </c>
       <c r="X36" s="134" t="n">
-        <v>700.0000000071039</v>
+        <v>875.0000000032207</v>
       </c>
       <c r="Y36" s="134" t="n">
-        <v>1100.000000002231</v>
+        <v>1375.000000001347</v>
       </c>
       <c r="Z36" s="134" t="n">
-        <v>1200</v>
+        <v>1500.000000005169</v>
       </c>
       <c r="AA36" s="134" t="n">
-        <v>700.0000000055021</v>
+        <v>875.0000000024945</v>
       </c>
       <c r="AB36" s="134" t="n">
-        <v>1100.000000001727</v>
+        <v>1375.000000001044</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -7253,70 +7253,70 @@
       </c>
       <c r="F37" s="123" t="inlineStr"/>
       <c r="G37" s="133" t="n">
-        <v>310.7645790319978</v>
+        <v>414.5423506083426</v>
       </c>
       <c r="H37" s="133" t="n">
-        <v>309.740854777321</v>
+        <v>413.5186263536663</v>
       </c>
       <c r="I37" s="134" t="n">
-        <v>757.8216299537</v>
+        <v>947.47493048312</v>
       </c>
       <c r="J37" s="134" t="n">
-        <v>455.2927785943799</v>
+        <v>569.3142583809845</v>
       </c>
       <c r="K37" s="134" t="n">
-        <v>726.5443341700756</v>
+        <v>908.3788890384991</v>
       </c>
       <c r="L37" s="134" t="n">
-        <v>756.8141744443094</v>
+        <v>946.4674749875754</v>
       </c>
       <c r="M37" s="134" t="n">
-        <v>454.2833269729815</v>
+        <v>568.3048067619046</v>
       </c>
       <c r="N37" s="134" t="n">
-        <v>725.5339346888293</v>
+        <v>907.3684895586309</v>
       </c>
       <c r="O37" s="134" t="n">
-        <v>757.030057770256</v>
+        <v>946.6833583101202</v>
       </c>
       <c r="P37" s="134" t="n">
-        <v>454.4996380358925</v>
+        <v>568.5211178241669</v>
       </c>
       <c r="Q37" s="134" t="n">
-        <v>725.7504488639092</v>
+        <v>907.5850037333259</v>
       </c>
       <c r="R37" s="133" t="n">
-        <v>310.7645790319978</v>
+        <v>414.5423506083426</v>
       </c>
       <c r="S37" s="133" t="n">
-        <v>309.740854777321</v>
+        <v>413.5186263536663</v>
       </c>
       <c r="T37" s="134" t="n">
-        <v>757.8216299537</v>
+        <v>947.47493048312</v>
       </c>
       <c r="U37" s="134" t="n">
-        <v>455.2927785943799</v>
+        <v>569.3142583809845</v>
       </c>
       <c r="V37" s="134" t="n">
-        <v>726.5443341700756</v>
+        <v>908.3788890384991</v>
       </c>
       <c r="W37" s="134" t="n">
-        <v>756.8141744443094</v>
+        <v>946.4674749875754</v>
       </c>
       <c r="X37" s="134" t="n">
-        <v>454.2833269729815</v>
+        <v>568.3048067619046</v>
       </c>
       <c r="Y37" s="134" t="n">
-        <v>725.5339346888293</v>
+        <v>907.3684895586309</v>
       </c>
       <c r="Z37" s="134" t="n">
-        <v>757.030057770256</v>
+        <v>946.6833583101202</v>
       </c>
       <c r="AA37" s="134" t="n">
-        <v>454.4996380358925</v>
+        <v>568.5211178241669</v>
       </c>
       <c r="AB37" s="134" t="n">
-        <v>725.7504488639092</v>
+        <v>907.5850037333259</v>
       </c>
     </row>
     <row r="38" ht="24" customHeight="1">
@@ -7347,70 +7347,70 @@
       </c>
       <c r="F38" s="123" t="inlineStr"/>
       <c r="G38" s="133" t="n">
-        <v>380.6655928127032</v>
+        <v>507.5362606554534</v>
       </c>
       <c r="H38" s="133" t="n">
-        <v>380.7620535247044</v>
+        <v>507.6327213674551</v>
       </c>
       <c r="I38" s="134" t="n">
-        <v>927.502479497927</v>
+        <v>1159.357919552818</v>
       </c>
       <c r="J38" s="134" t="n">
-        <v>557.6541311411593</v>
+        <v>697.047963454307</v>
       </c>
       <c r="K38" s="134" t="n">
-        <v>889.265279526212</v>
+        <v>1111.562126554527</v>
       </c>
       <c r="L38" s="134" t="n">
-        <v>927.6052130907536</v>
+        <v>1159.460653162571</v>
       </c>
       <c r="M38" s="134" t="n">
-        <v>557.7544244420073</v>
+        <v>697.1482567579897</v>
       </c>
       <c r="N38" s="134" t="n">
-        <v>889.3644140470044</v>
+        <v>1111.661261077004</v>
       </c>
       <c r="O38" s="134" t="n">
-        <v>927.583198752497</v>
+        <v>1159.438638820156</v>
       </c>
       <c r="P38" s="134" t="n">
-        <v>557.732933021843</v>
+        <v>697.1267653370321</v>
       </c>
       <c r="Q38" s="134" t="n">
-        <v>889.3431709360505</v>
+        <v>1111.640017965579</v>
       </c>
       <c r="R38" s="133" t="n">
-        <v>380.6655928127032</v>
+        <v>507.5362606554534</v>
       </c>
       <c r="S38" s="133" t="n">
-        <v>380.7620535247044</v>
+        <v>507.6327213674551</v>
       </c>
       <c r="T38" s="134" t="n">
-        <v>927.502479497927</v>
+        <v>1159.357919552818</v>
       </c>
       <c r="U38" s="134" t="n">
-        <v>557.6541311411593</v>
+        <v>697.047963454307</v>
       </c>
       <c r="V38" s="134" t="n">
-        <v>889.265279526212</v>
+        <v>1111.562126554527</v>
       </c>
       <c r="W38" s="134" t="n">
-        <v>927.6052130907536</v>
+        <v>1159.460653162571</v>
       </c>
       <c r="X38" s="134" t="n">
-        <v>557.7544244420073</v>
+        <v>697.1482567579897</v>
       </c>
       <c r="Y38" s="134" t="n">
-        <v>889.3644140470044</v>
+        <v>1111.661261077004</v>
       </c>
       <c r="Z38" s="134" t="n">
-        <v>927.583198752497</v>
+        <v>1159.438638820156</v>
       </c>
       <c r="AA38" s="134" t="n">
-        <v>557.732933021843</v>
+        <v>697.1267653370321</v>
       </c>
       <c r="AB38" s="134" t="n">
-        <v>889.3431709360505</v>
+        <v>1111.640017965579</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -7539,70 +7539,70 @@
         </is>
       </c>
       <c r="G40" s="136" t="n">
-        <v>247.621178511552</v>
+        <v>330.3126299668069</v>
       </c>
       <c r="H40" s="136" t="n">
-        <v>246.805461973961</v>
+        <v>329.4969134292162</v>
       </c>
       <c r="I40" s="137" t="n">
-        <v>603.8419362180877</v>
+        <v>754.9601039706135</v>
       </c>
       <c r="J40" s="137" t="n">
-        <v>362.7830905134501</v>
+        <v>453.6368592677167</v>
       </c>
       <c r="K40" s="137" t="n">
-        <v>578.9197881833272</v>
+        <v>723.8078797119515</v>
       </c>
       <c r="L40" s="137" t="n">
-        <v>603.039182824151</v>
+        <v>754.1573505877096</v>
       </c>
       <c r="M40" s="137" t="n">
-        <v>361.9787465920171</v>
+        <v>452.8325153481312</v>
       </c>
       <c r="N40" s="137" t="n">
-        <v>578.114688995083</v>
+        <v>723.0027805248055</v>
       </c>
       <c r="O40" s="137" t="n">
-        <v>603.2112014105625</v>
+        <v>754.3293691714105</v>
       </c>
       <c r="P40" s="137" t="n">
-        <v>362.1511060046952</v>
+        <v>453.0048747602923</v>
       </c>
       <c r="Q40" s="137" t="n">
-        <v>578.2872102501269</v>
+        <v>723.1753017795427</v>
       </c>
       <c r="R40" s="136" t="n">
-        <v>247.621178511552</v>
+        <v>330.3126299668069</v>
       </c>
       <c r="S40" s="136" t="n">
-        <v>246.805461973961</v>
+        <v>329.4969134292162</v>
       </c>
       <c r="T40" s="137" t="n">
-        <v>603.8419362180877</v>
+        <v>754.9601039706135</v>
       </c>
       <c r="U40" s="137" t="n">
-        <v>362.7830905134501</v>
+        <v>453.6368592677167</v>
       </c>
       <c r="V40" s="137" t="n">
-        <v>578.9197881833272</v>
+        <v>723.8078797119515</v>
       </c>
       <c r="W40" s="137" t="n">
-        <v>603.039182824151</v>
+        <v>754.1573505877096</v>
       </c>
       <c r="X40" s="137" t="n">
-        <v>361.9787465920171</v>
+        <v>452.8325153481312</v>
       </c>
       <c r="Y40" s="137" t="n">
-        <v>578.114688995083</v>
+        <v>723.0027805248055</v>
       </c>
       <c r="Z40" s="137" t="n">
-        <v>603.2112014105625</v>
+        <v>754.3293691714105</v>
       </c>
       <c r="AA40" s="137" t="n">
-        <v>362.1511060046952</v>
+        <v>453.0048747602923</v>
       </c>
       <c r="AB40" s="137" t="n">
-        <v>578.2872102501269</v>
+        <v>723.1753017795427</v>
       </c>
     </row>
     <row r="41" ht="24" customHeight="1">
@@ -9203,70 +9203,70 @@
       </c>
       <c r="F59" s="123" t="inlineStr"/>
       <c r="G59" s="126" t="n">
-        <v>435070.4106447972</v>
+        <v>580359.2908516801</v>
       </c>
       <c r="H59" s="126" t="n">
-        <v>154870.4273886605</v>
+        <v>206759.3131768332</v>
       </c>
       <c r="I59" s="126" t="n">
-        <v>757821.6299537</v>
+        <v>947474.93048312</v>
       </c>
       <c r="J59" s="126" t="n">
-        <v>455292.7785943799</v>
+        <v>569314.2583809845</v>
       </c>
       <c r="K59" s="126" t="n">
-        <v>726544.3341700756</v>
+        <v>908378.8890384991</v>
       </c>
       <c r="L59" s="126" t="n">
-        <v>332998.2367554961</v>
+        <v>416445.6889945332</v>
       </c>
       <c r="M59" s="126" t="n">
-        <v>199884.6638681118</v>
+        <v>250054.114975238</v>
       </c>
       <c r="N59" s="126" t="n">
-        <v>319234.9312630849</v>
+        <v>399242.1354057976</v>
       </c>
       <c r="O59" s="126" t="n">
-        <v>378515.028885128</v>
+        <v>473341.6791550601</v>
       </c>
       <c r="P59" s="126" t="n">
-        <v>227249.8190179462</v>
+        <v>284260.5589120834</v>
       </c>
       <c r="Q59" s="126" t="n">
-        <v>362875.2244319546</v>
+        <v>453792.501866663</v>
       </c>
       <c r="R59" s="126" t="n">
-        <v>435070.4106447972</v>
+        <v>580359.2908516801</v>
       </c>
       <c r="S59" s="126" t="n">
-        <v>154870.4273886605</v>
+        <v>206759.3131768332</v>
       </c>
       <c r="T59" s="126" t="n">
-        <v>757821.6299537</v>
+        <v>947474.93048312</v>
       </c>
       <c r="U59" s="126" t="n">
-        <v>455292.7785943799</v>
+        <v>569314.2583809845</v>
       </c>
       <c r="V59" s="126" t="n">
-        <v>726544.3341700756</v>
+        <v>908378.8890384991</v>
       </c>
       <c r="W59" s="126" t="n">
-        <v>332998.2367554961</v>
+        <v>416445.6889945332</v>
       </c>
       <c r="X59" s="126" t="n">
-        <v>199884.6638681118</v>
+        <v>250054.114975238</v>
       </c>
       <c r="Y59" s="126" t="n">
-        <v>319234.9312630849</v>
+        <v>399242.1354057976</v>
       </c>
       <c r="Z59" s="126" t="n">
-        <v>378515.028885128</v>
+        <v>473341.6791550601</v>
       </c>
       <c r="AA59" s="126" t="n">
-        <v>227249.8190179462</v>
+        <v>284260.5589120834</v>
       </c>
       <c r="AB59" s="126" t="n">
-        <v>362875.2244319546</v>
+        <v>453792.501866663</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
@@ -9485,70 +9485,70 @@
       </c>
       <c r="F62" s="123" t="inlineStr"/>
       <c r="G62" s="126" t="n">
-        <v>76981.6492033269</v>
+        <v>102628.4154867779</v>
       </c>
       <c r="H62" s="126" t="n">
-        <v>27520.02851381328</v>
+        <v>36679.5879007601</v>
       </c>
       <c r="I62" s="126" t="n">
-        <v>133954.5233663569</v>
+        <v>167432.611067474</v>
       </c>
       <c r="J62" s="126" t="n">
-        <v>80551.35353143782</v>
+        <v>100678.7179877973</v>
       </c>
       <c r="K62" s="126" t="n">
-        <v>128433.3747843129</v>
+        <v>160531.2774202566</v>
       </c>
       <c r="L62" s="126" t="n">
-        <v>58963.60691368263</v>
+        <v>73693.96550324962</v>
       </c>
       <c r="M62" s="126" t="n">
-        <v>35466.05714843821</v>
+        <v>44322.09750941646</v>
       </c>
       <c r="N62" s="126" t="n">
-        <v>56534.07287949516</v>
+        <v>70657.15003941741</v>
       </c>
       <c r="O62" s="126" t="n">
-        <v>66998.3479624046</v>
+        <v>83737.39181388501</v>
       </c>
       <c r="P62" s="126" t="n">
-        <v>40296.6246181497</v>
+        <v>50360.30684647681</v>
       </c>
       <c r="Q62" s="126" t="n">
-        <v>64237.56951220073</v>
+        <v>80286.52083026024</v>
       </c>
       <c r="R62" s="126" t="n">
-        <v>76981.6492033269</v>
+        <v>102628.4154867779</v>
       </c>
       <c r="S62" s="126" t="n">
-        <v>27520.02851381328</v>
+        <v>36679.5879007601</v>
       </c>
       <c r="T62" s="126" t="n">
-        <v>133954.5233663569</v>
+        <v>167432.611067474</v>
       </c>
       <c r="U62" s="126" t="n">
-        <v>80551.35353143782</v>
+        <v>100678.7179877973</v>
       </c>
       <c r="V62" s="126" t="n">
-        <v>128433.3747843129</v>
+        <v>160531.2774202566</v>
       </c>
       <c r="W62" s="126" t="n">
-        <v>58963.60691368263</v>
+        <v>73693.96550324962</v>
       </c>
       <c r="X62" s="126" t="n">
-        <v>35466.05714843821</v>
+        <v>44322.09750941646</v>
       </c>
       <c r="Y62" s="126" t="n">
-        <v>56534.07287949516</v>
+        <v>70657.15003941741</v>
       </c>
       <c r="Z62" s="126" t="n">
-        <v>66998.3479624046</v>
+        <v>83737.39181388501</v>
       </c>
       <c r="AA62" s="126" t="n">
-        <v>40296.6246181497</v>
+        <v>50360.30684647681</v>
       </c>
       <c r="AB62" s="126" t="n">
-        <v>64237.56951220073</v>
+        <v>80286.52083026024</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
@@ -9579,70 +9579,70 @@
       </c>
       <c r="F63" s="123" t="inlineStr"/>
       <c r="G63" s="126" t="n">
-        <v>20053.56008966067</v>
+        <v>26736.84857917728</v>
       </c>
       <c r="H63" s="126" t="n">
-        <v>7164.360859878385</v>
+        <v>9551.249606134326</v>
       </c>
       <c r="I63" s="126" t="n">
-        <v>34900.1161778702</v>
+        <v>43624.16800222352</v>
       </c>
       <c r="J63" s="126" t="n">
-        <v>20983.78901534147</v>
+        <v>26228.77708552528</v>
       </c>
       <c r="K63" s="126" t="n">
-        <v>33461.36057182348</v>
+        <v>41825.75009577096</v>
       </c>
       <c r="L63" s="126" t="n">
-        <v>15358.24009075282</v>
+        <v>19196.82289374853</v>
       </c>
       <c r="M63" s="126" t="n">
-        <v>9235.015737933145</v>
+        <v>11542.81048886095</v>
       </c>
       <c r="N63" s="126" t="n">
-        <v>14725.1280381019</v>
+        <v>18405.45942866669</v>
       </c>
       <c r="O63" s="126" t="n">
-        <v>17452.01252871589</v>
+        <v>21814.03844113276</v>
       </c>
       <c r="P63" s="126" t="n">
-        <v>10493.81287482553</v>
+        <v>13116.30690995584</v>
       </c>
       <c r="Q63" s="126" t="n">
-        <v>16732.58152386991</v>
+        <v>20914.7762858665</v>
       </c>
       <c r="R63" s="126" t="n">
-        <v>20053.56008966067</v>
+        <v>26736.84857917728</v>
       </c>
       <c r="S63" s="126" t="n">
-        <v>7164.360859878385</v>
+        <v>9551.249606134326</v>
       </c>
       <c r="T63" s="126" t="n">
-        <v>34900.1161778702</v>
+        <v>43624.16800222352</v>
       </c>
       <c r="U63" s="126" t="n">
-        <v>20983.78901534147</v>
+        <v>26228.77708552528</v>
       </c>
       <c r="V63" s="126" t="n">
-        <v>33461.36057182348</v>
+        <v>41825.75009577096</v>
       </c>
       <c r="W63" s="126" t="n">
-        <v>15358.24009075282</v>
+        <v>19196.82289374853</v>
       </c>
       <c r="X63" s="126" t="n">
-        <v>9235.015737933145</v>
+        <v>11542.81048886095</v>
       </c>
       <c r="Y63" s="126" t="n">
-        <v>14725.1280381019</v>
+        <v>18405.45942866669</v>
       </c>
       <c r="Z63" s="126" t="n">
-        <v>17452.01252871589</v>
+        <v>21814.03844113276</v>
       </c>
       <c r="AA63" s="126" t="n">
-        <v>10493.81287482553</v>
+        <v>13116.30690995584</v>
       </c>
       <c r="AB63" s="126" t="n">
-        <v>16732.58152386991</v>
+        <v>20914.7762858665</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
@@ -9673,70 +9673,70 @@
       </c>
       <c r="F64" s="123" t="inlineStr"/>
       <c r="G64" s="126" t="n">
-        <v>37891.91776882572</v>
+        <v>50544.84852129683</v>
       </c>
       <c r="H64" s="126" t="n">
-        <v>13489.8370319167</v>
+        <v>18008.74087208496</v>
       </c>
       <c r="I64" s="126" t="n">
-        <v>65999.70428611556</v>
+        <v>82516.24756980907</v>
       </c>
       <c r="J64" s="126" t="n">
-        <v>39653.04512387666</v>
+        <v>49582.95776398968</v>
       </c>
       <c r="K64" s="126" t="n">
-        <v>63275.82440548581</v>
+        <v>79111.44808074881</v>
       </c>
       <c r="L64" s="126" t="n">
-        <v>29002.64732957065</v>
+        <v>36269.92637492636</v>
       </c>
       <c r="M64" s="126" t="n">
-        <v>17410.04080965132</v>
+        <v>21779.2023713899</v>
       </c>
       <c r="N64" s="126" t="n">
-        <v>27804.02737274662</v>
+        <v>34771.70178991518</v>
       </c>
       <c r="O64" s="126" t="n">
-        <v>32966.617717881</v>
+        <v>41224.88936018253</v>
       </c>
       <c r="P64" s="126" t="n">
-        <v>19793.21984336982</v>
+        <v>24758.17616349904</v>
       </c>
       <c r="Q64" s="126" t="n">
-        <v>31604.57705484878</v>
+        <v>39522.38889252355</v>
       </c>
       <c r="R64" s="126" t="n">
-        <v>37891.91776882572</v>
+        <v>50544.84852129683</v>
       </c>
       <c r="S64" s="126" t="n">
-        <v>13489.8370319167</v>
+        <v>18008.74087208496</v>
       </c>
       <c r="T64" s="126" t="n">
-        <v>65999.70428611556</v>
+        <v>82516.24756980907</v>
       </c>
       <c r="U64" s="126" t="n">
-        <v>39653.04512387666</v>
+        <v>49582.95776398968</v>
       </c>
       <c r="V64" s="126" t="n">
-        <v>63275.82440548581</v>
+        <v>79111.44808074881</v>
       </c>
       <c r="W64" s="126" t="n">
-        <v>29002.64732957065</v>
+        <v>36269.92637492636</v>
       </c>
       <c r="X64" s="126" t="n">
-        <v>17410.04080965132</v>
+        <v>21779.2023713899</v>
       </c>
       <c r="Y64" s="126" t="n">
-        <v>27804.02737274662</v>
+        <v>34771.70178991518</v>
       </c>
       <c r="Z64" s="126" t="n">
-        <v>32966.617717881</v>
+        <v>41224.88936018253</v>
       </c>
       <c r="AA64" s="126" t="n">
-        <v>19793.21984336982</v>
+        <v>24758.17616349904</v>
       </c>
       <c r="AB64" s="126" t="n">
-        <v>31604.57705484878</v>
+        <v>39522.38889252355</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
@@ -9767,70 +9767,70 @@
       </c>
       <c r="F65" s="123" t="inlineStr"/>
       <c r="G65" s="126" t="n">
-        <v>11108.31234256933</v>
+        <v>14811.0831234257</v>
       </c>
       <c r="H65" s="126" t="n">
-        <v>3967.254408060466</v>
+        <v>5289.672544080604</v>
       </c>
       <c r="I65" s="126" t="n">
-        <v>122830.4167780296</v>
+        <v>153539.6743896757</v>
       </c>
       <c r="J65" s="126" t="n">
-        <v>52394.35660067869</v>
+        <v>65494.04242620258</v>
       </c>
       <c r="K65" s="126" t="n">
-        <v>67241.38235307336</v>
+        <v>84052.56024733675</v>
       </c>
       <c r="L65" s="126" t="n">
-        <v>54041.67973966443</v>
+        <v>67553.75308367999</v>
       </c>
       <c r="M65" s="126" t="n">
-        <v>23051.06035763631</v>
+        <v>28814.92211804088</v>
       </c>
       <c r="N65" s="126" t="n">
-        <v>29584.34387253252</v>
+        <v>36981.26214483411</v>
       </c>
       <c r="O65" s="126" t="n">
-        <v>61411.90156313884</v>
+        <v>76766.53036481881</v>
       </c>
       <c r="P65" s="126" t="n">
-        <v>26194.98495407817</v>
+        <v>32744.8278645272</v>
       </c>
       <c r="Q65" s="126" t="n">
-        <v>33619.02656644283</v>
+        <v>42024.61551261343</v>
       </c>
       <c r="R65" s="126" t="n">
-        <v>11108.31234256933</v>
+        <v>14811.0831234257</v>
       </c>
       <c r="S65" s="126" t="n">
-        <v>3967.254408060466</v>
+        <v>5289.672544080604</v>
       </c>
       <c r="T65" s="126" t="n">
-        <v>122830.4167780296</v>
+        <v>153539.6743896757</v>
       </c>
       <c r="U65" s="126" t="n">
-        <v>52394.35660067869</v>
+        <v>65494.04242620258</v>
       </c>
       <c r="V65" s="126" t="n">
-        <v>67241.38235307336</v>
+        <v>84052.56024733675</v>
       </c>
       <c r="W65" s="126" t="n">
-        <v>54041.67973966443</v>
+        <v>67553.75308367999</v>
       </c>
       <c r="X65" s="126" t="n">
-        <v>23051.06035763631</v>
+        <v>28814.92211804088</v>
       </c>
       <c r="Y65" s="126" t="n">
-        <v>29584.34387253252</v>
+        <v>36981.26214483411</v>
       </c>
       <c r="Z65" s="126" t="n">
-        <v>61411.90156313884</v>
+        <v>76766.53036481881</v>
       </c>
       <c r="AA65" s="126" t="n">
-        <v>26194.98495407817</v>
+        <v>32744.8278645272</v>
       </c>
       <c r="AB65" s="126" t="n">
-        <v>33619.02656644283</v>
+        <v>42024.61551261343</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
@@ -9861,70 +9861,70 @@
       </c>
       <c r="F66" s="123" t="inlineStr"/>
       <c r="G66" s="126" t="n">
-        <v>47988.26629412113</v>
+        <v>64013.62978094031</v>
       </c>
       <c r="H66" s="126" t="n">
-        <v>17082.20814096925</v>
+        <v>22805.55224340469</v>
       </c>
       <c r="I66" s="126" t="n">
-        <v>83587.72578389311</v>
+        <v>104506.4848322881</v>
       </c>
       <c r="J66" s="126" t="n">
-        <v>50218.7934789601</v>
+        <v>62795.36269942258</v>
       </c>
       <c r="K66" s="126" t="n">
-        <v>80137.84005895934</v>
+        <v>100194.1914609464</v>
       </c>
       <c r="L66" s="126" t="n">
-        <v>36729.70551413122</v>
+        <v>45933.95949609701</v>
       </c>
       <c r="M66" s="126" t="n">
-        <v>22047.27842465274</v>
+        <v>27580.96888176876</v>
       </c>
       <c r="N66" s="126" t="n">
-        <v>35211.61291831826</v>
+        <v>44036.40753525947</v>
       </c>
       <c r="O66" s="126" t="n">
-        <v>41750.20768602961</v>
+        <v>52209.58721080312</v>
       </c>
       <c r="P66" s="126" t="n">
-        <v>25065.65503767947</v>
+        <v>31353.9396480028</v>
       </c>
       <c r="Q66" s="126" t="n">
-        <v>40025.13725484459</v>
+        <v>50053.31295589292</v>
       </c>
       <c r="R66" s="126" t="n">
-        <v>47988.26629412113</v>
+        <v>64013.62978094031</v>
       </c>
       <c r="S66" s="126" t="n">
-        <v>17082.20814096925</v>
+        <v>22805.55224340469</v>
       </c>
       <c r="T66" s="126" t="n">
-        <v>83587.72578389311</v>
+        <v>104506.4848322881</v>
       </c>
       <c r="U66" s="126" t="n">
-        <v>50218.7934789601</v>
+        <v>62795.36269942258</v>
       </c>
       <c r="V66" s="126" t="n">
-        <v>80137.84005895934</v>
+        <v>100194.1914609464</v>
       </c>
       <c r="W66" s="126" t="n">
-        <v>36729.70551413122</v>
+        <v>45933.95949609701</v>
       </c>
       <c r="X66" s="126" t="n">
-        <v>22047.27842465274</v>
+        <v>27580.96888176876</v>
       </c>
       <c r="Y66" s="126" t="n">
-        <v>35211.61291831826</v>
+        <v>44036.40753525947</v>
       </c>
       <c r="Z66" s="126" t="n">
-        <v>41750.20768602961</v>
+        <v>52209.58721080312</v>
       </c>
       <c r="AA66" s="126" t="n">
-        <v>25065.65503767947</v>
+        <v>31353.9396480028</v>
       </c>
       <c r="AB66" s="126" t="n">
-        <v>40025.13725484459</v>
+        <v>50053.31295589292</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
@@ -9955,70 +9955,70 @@
       </c>
       <c r="F67" s="123" t="inlineStr"/>
       <c r="G67" s="126" t="n">
-        <v>630000.0000000031</v>
+        <v>840000.0000000003</v>
       </c>
       <c r="H67" s="126" t="n">
-        <v>225000.0000000008</v>
+        <v>299999.9999999999</v>
       </c>
       <c r="I67" s="126" t="n">
-        <v>1200000.000002668</v>
+        <v>1500000.000001293</v>
       </c>
       <c r="J67" s="126" t="n">
-        <v>700000.0000013767</v>
+        <v>875000.000000624</v>
       </c>
       <c r="K67" s="126" t="n">
-        <v>1100000.000000433</v>
+        <v>1375000.000000261</v>
       </c>
       <c r="L67" s="126" t="n">
-        <v>528000</v>
+        <v>660000.0000029369</v>
       </c>
       <c r="M67" s="126" t="n">
-        <v>308000.0000031258</v>
+        <v>385000.0000014171</v>
       </c>
       <c r="N67" s="126" t="n">
-        <v>484000.0000009815</v>
+        <v>605000.0000005927</v>
       </c>
       <c r="O67" s="126" t="n">
-        <v>600000</v>
+        <v>750000.0000025844</v>
       </c>
       <c r="P67" s="126" t="n">
-        <v>350000.0000027511</v>
+        <v>437500.0000012473</v>
       </c>
       <c r="Q67" s="126" t="n">
-        <v>550000.0000008636</v>
+        <v>687500.0000005218</v>
       </c>
       <c r="R67" s="126" t="n">
-        <v>630000.0000000031</v>
+        <v>840000.0000000003</v>
       </c>
       <c r="S67" s="126" t="n">
-        <v>225000.0000000008</v>
+        <v>299999.9999999999</v>
       </c>
       <c r="T67" s="126" t="n">
-        <v>1200000.000002668</v>
+        <v>1500000.000001293</v>
       </c>
       <c r="U67" s="126" t="n">
-        <v>700000.0000013767</v>
+        <v>875000.000000624</v>
       </c>
       <c r="V67" s="126" t="n">
-        <v>1100000.000000433</v>
+        <v>1375000.000000261</v>
       </c>
       <c r="W67" s="126" t="n">
-        <v>528000</v>
+        <v>660000.0000029369</v>
       </c>
       <c r="X67" s="126" t="n">
-        <v>308000.0000031258</v>
+        <v>385000.0000014171</v>
       </c>
       <c r="Y67" s="126" t="n">
-        <v>484000.0000009815</v>
+        <v>605000.0000005927</v>
       </c>
       <c r="Z67" s="126" t="n">
-        <v>600000</v>
+        <v>750000.0000025844</v>
       </c>
       <c r="AA67" s="126" t="n">
-        <v>350000.0000027511</v>
+        <v>437500.0000012473</v>
       </c>
       <c r="AB67" s="126" t="n">
-        <v>550000.0000008636</v>
+        <v>687500.0000005218</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
@@ -10049,70 +10049,70 @@
       </c>
       <c r="F68" s="123" t="inlineStr"/>
       <c r="G68" s="126" t="n">
-        <v>441000.0000000022</v>
+        <v>588000.0000000002</v>
       </c>
       <c r="H68" s="126" t="n">
-        <v>157500.0000000005</v>
+        <v>210000</v>
       </c>
       <c r="I68" s="126" t="n">
-        <v>840000.0000018671</v>
+        <v>1050000.000000905</v>
       </c>
       <c r="J68" s="126" t="n">
-        <v>490000.0000009636</v>
+        <v>612500.0000004368</v>
       </c>
       <c r="K68" s="126" t="n">
-        <v>770000.0000003028</v>
+        <v>962500.0000001823</v>
       </c>
       <c r="L68" s="126" t="n">
-        <v>369600</v>
+        <v>462000.0000020558</v>
       </c>
       <c r="M68" s="126" t="n">
-        <v>215600.000002188</v>
+        <v>269500.000000992</v>
       </c>
       <c r="N68" s="126" t="n">
-        <v>338800.000000687</v>
+        <v>423500.0000004149</v>
       </c>
       <c r="O68" s="126" t="n">
-        <v>420000</v>
+        <v>525000.0000018091</v>
       </c>
       <c r="P68" s="126" t="n">
-        <v>245000.0000019257</v>
+        <v>306250.0000008731</v>
       </c>
       <c r="Q68" s="126" t="n">
-        <v>385000.0000006044</v>
+        <v>481250.0000003652</v>
       </c>
       <c r="R68" s="126" t="n">
-        <v>441000.0000000022</v>
+        <v>588000.0000000002</v>
       </c>
       <c r="S68" s="126" t="n">
-        <v>157500.0000000005</v>
+        <v>210000</v>
       </c>
       <c r="T68" s="126" t="n">
-        <v>840000.0000018671</v>
+        <v>1050000.000000905</v>
       </c>
       <c r="U68" s="126" t="n">
-        <v>490000.0000009636</v>
+        <v>612500.0000004368</v>
       </c>
       <c r="V68" s="126" t="n">
-        <v>770000.0000003028</v>
+        <v>962500.0000001823</v>
       </c>
       <c r="W68" s="126" t="n">
-        <v>369600</v>
+        <v>462000.0000020558</v>
       </c>
       <c r="X68" s="126" t="n">
-        <v>215600.000002188</v>
+        <v>269500.000000992</v>
       </c>
       <c r="Y68" s="126" t="n">
-        <v>338800.000000687</v>
+        <v>423500.0000004149</v>
       </c>
       <c r="Z68" s="126" t="n">
-        <v>420000</v>
+        <v>525000.0000018091</v>
       </c>
       <c r="AA68" s="126" t="n">
-        <v>245000.0000019257</v>
+        <v>306250.0000008731</v>
       </c>
       <c r="AB68" s="126" t="n">
-        <v>385000.0000006044</v>
+        <v>481250.0000003652</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
@@ -10143,70 +10143,70 @@
       </c>
       <c r="F69" s="123" t="inlineStr"/>
       <c r="G69" s="126" t="n">
-        <v>189000.000000001</v>
+        <v>252000.0000000002</v>
       </c>
       <c r="H69" s="126" t="n">
-        <v>67500.00000000022</v>
+        <v>90000</v>
       </c>
       <c r="I69" s="126" t="n">
-        <v>360000.0000008002</v>
+        <v>450000.0000003878</v>
       </c>
       <c r="J69" s="126" t="n">
-        <v>210000.000000413</v>
+        <v>262500.0000001873</v>
       </c>
       <c r="K69" s="126" t="n">
-        <v>330000.0000001298</v>
+        <v>412500.0000000783</v>
       </c>
       <c r="L69" s="126" t="n">
-        <v>158400</v>
+        <v>198000.0000008811</v>
       </c>
       <c r="M69" s="126" t="n">
-        <v>92400.00000093774</v>
+        <v>115500.0000004251</v>
       </c>
       <c r="N69" s="126" t="n">
-        <v>145200.0000002945</v>
+        <v>181500.0000001778</v>
       </c>
       <c r="O69" s="126" t="n">
-        <v>180000</v>
+        <v>225000.0000007753</v>
       </c>
       <c r="P69" s="126" t="n">
-        <v>105000.0000008253</v>
+        <v>131250.0000003742</v>
       </c>
       <c r="Q69" s="126" t="n">
-        <v>165000.0000002591</v>
+        <v>206250.0000001566</v>
       </c>
       <c r="R69" s="126" t="n">
-        <v>189000.000000001</v>
+        <v>252000.0000000002</v>
       </c>
       <c r="S69" s="126" t="n">
-        <v>67500.00000000022</v>
+        <v>90000</v>
       </c>
       <c r="T69" s="126" t="n">
-        <v>360000.0000008002</v>
+        <v>450000.0000003878</v>
       </c>
       <c r="U69" s="126" t="n">
-        <v>210000.000000413</v>
+        <v>262500.0000001873</v>
       </c>
       <c r="V69" s="126" t="n">
-        <v>330000.0000001298</v>
+        <v>412500.0000000783</v>
       </c>
       <c r="W69" s="126" t="n">
-        <v>158400</v>
+        <v>198000.0000008811</v>
       </c>
       <c r="X69" s="126" t="n">
-        <v>92400.00000093774</v>
+        <v>115500.0000004251</v>
       </c>
       <c r="Y69" s="126" t="n">
-        <v>145200.0000002945</v>
+        <v>181500.0000001778</v>
       </c>
       <c r="Z69" s="126" t="n">
-        <v>180000</v>
+        <v>225000.0000007753</v>
       </c>
       <c r="AA69" s="126" t="n">
-        <v>105000.0000008253</v>
+        <v>131250.0000003742</v>
       </c>
       <c r="AB69" s="126" t="n">
-        <v>165000.0000002591</v>
+        <v>206250.0000001566</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
@@ -10237,70 +10237,70 @@
       </c>
       <c r="F70" s="123" t="inlineStr"/>
       <c r="G70" s="126" t="n">
-        <v>630000.0000000031</v>
+        <v>840000.0000000005</v>
       </c>
       <c r="H70" s="126" t="n">
-        <v>225000.0000000008</v>
+        <v>300000</v>
       </c>
       <c r="I70" s="126" t="n">
-        <v>1200000.000002667</v>
+        <v>1500000.000001292</v>
       </c>
       <c r="J70" s="126" t="n">
-        <v>700000.0000013766</v>
+        <v>875000.000000624</v>
       </c>
       <c r="K70" s="126" t="n">
-        <v>1100000.000000433</v>
+        <v>1375000.000000261</v>
       </c>
       <c r="L70" s="126" t="n">
-        <v>528000</v>
+        <v>660000.0000029369</v>
       </c>
       <c r="M70" s="126" t="n">
-        <v>308000.0000031258</v>
+        <v>385000.0000014171</v>
       </c>
       <c r="N70" s="126" t="n">
-        <v>484000.0000009814</v>
+        <v>605000.0000005928</v>
       </c>
       <c r="O70" s="126" t="n">
-        <v>600000</v>
+        <v>750000.0000025844</v>
       </c>
       <c r="P70" s="126" t="n">
-        <v>350000.0000027511</v>
+        <v>437500.0000012473</v>
       </c>
       <c r="Q70" s="126" t="n">
-        <v>550000.0000008636</v>
+        <v>687500.0000005218</v>
       </c>
       <c r="R70" s="126" t="n">
-        <v>630000.0000000031</v>
+        <v>840000.0000000005</v>
       </c>
       <c r="S70" s="126" t="n">
-        <v>225000.0000000008</v>
+        <v>300000</v>
       </c>
       <c r="T70" s="126" t="n">
-        <v>1200000.000002667</v>
+        <v>1500000.000001292</v>
       </c>
       <c r="U70" s="126" t="n">
-        <v>700000.0000013766</v>
+        <v>875000.000000624</v>
       </c>
       <c r="V70" s="126" t="n">
-        <v>1100000.000000433</v>
+        <v>1375000.000000261</v>
       </c>
       <c r="W70" s="126" t="n">
-        <v>528000</v>
+        <v>660000.0000029369</v>
       </c>
       <c r="X70" s="126" t="n">
-        <v>308000.0000031258</v>
+        <v>385000.0000014171</v>
       </c>
       <c r="Y70" s="126" t="n">
-        <v>484000.0000009814</v>
+        <v>605000.0000005928</v>
       </c>
       <c r="Z70" s="126" t="n">
-        <v>600000</v>
+        <v>750000.0000025844</v>
       </c>
       <c r="AA70" s="126" t="n">
-        <v>350000.0000027511</v>
+        <v>437500.0000012473</v>
       </c>
       <c r="AB70" s="126" t="n">
-        <v>550000.0000008636</v>
+        <v>687500.0000005218</v>
       </c>
     </row>
     <row r="72">
@@ -10659,70 +10659,70 @@
       </c>
       <c r="F76" s="123" t="inlineStr"/>
       <c r="G76" s="141" t="n">
-        <v>0.0811717235790007</v>
+        <v>0.06087983948007971</v>
       </c>
       <c r="H76" s="141" t="n">
-        <v>0.0676584939577328</v>
+        <v>0.05074631332083004</v>
       </c>
       <c r="I76" s="141" t="n">
-        <v>0.02777098792146538</v>
+        <v>0.02221699321089768</v>
       </c>
       <c r="J76" s="141" t="n">
-        <v>0.05493391116475157</v>
+        <v>0.0439477661902375</v>
       </c>
       <c r="K76" s="141" t="n">
-        <v>0.0419056837595459</v>
+        <v>0.03352484497967969</v>
       </c>
       <c r="L76" s="141" t="n">
-        <v>0.02776937426272354</v>
+        <v>0.02221596043811579</v>
       </c>
       <c r="M76" s="141" t="n">
-        <v>0.05492884260592908</v>
+        <v>0.04394452215847597</v>
       </c>
       <c r="N76" s="141" t="n">
-        <v>0.04190331368273124</v>
+        <v>0.03352332808634563</v>
       </c>
       <c r="O76" s="141" t="n">
-        <v>0.02776972003086109</v>
+        <v>0.02221618173843729</v>
       </c>
       <c r="P76" s="141" t="n">
-        <v>0.05492992864679443</v>
+        <v>0.04394521726774178</v>
       </c>
       <c r="Q76" s="141" t="n">
-        <v>0.04190382153373486</v>
+        <v>0.03352365312334513</v>
       </c>
       <c r="R76" s="141" t="n">
-        <v>0.08162213373687528</v>
+        <v>0.06121765290700435</v>
       </c>
       <c r="S76" s="141" t="n">
-        <v>0.08161203015971229</v>
+        <v>0.0612119692735261</v>
       </c>
       <c r="T76" s="141" t="n">
-        <v>0.03264932634316756</v>
+        <v>0.02611969958569126</v>
       </c>
       <c r="U76" s="141" t="n">
-        <v>0.07319036890307866</v>
+        <v>0.05855314416413949</v>
       </c>
       <c r="V76" s="141" t="n">
-        <v>0.05157309162767646</v>
+        <v>0.04125884001467503</v>
       </c>
       <c r="W76" s="141" t="n">
-        <v>0.03264742922409431</v>
+        <v>0.02611848539281885</v>
       </c>
       <c r="X76" s="141" t="n">
-        <v>0.07318361588509471</v>
+        <v>0.05854882202729678</v>
       </c>
       <c r="Y76" s="141" t="n">
-        <v>0.05157017478733976</v>
+        <v>0.04125697318249647</v>
       </c>
       <c r="Z76" s="141" t="n">
-        <v>0.03264783573094217</v>
+        <v>0.02611874556744557</v>
       </c>
       <c r="AA76" s="141" t="n">
-        <v>0.0731850628552793</v>
+        <v>0.05854974814565452</v>
       </c>
       <c r="AB76" s="141" t="n">
-        <v>0.05157079979674167</v>
+        <v>0.04125737320372161</v>
       </c>
     </row>
     <row r="77" ht="24" customHeight="1">
@@ -10753,70 +10753,70 @@
       </c>
       <c r="F77" s="123" t="inlineStr"/>
       <c r="G77" s="139" t="n">
-        <v>13.5</v>
+        <v>18</v>
       </c>
       <c r="H77" s="139" t="n">
-        <v>13.5</v>
+        <v>18</v>
       </c>
       <c r="I77" s="139" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="J77" s="139" t="n">
-        <v>21</v>
+        <v>26.25</v>
       </c>
       <c r="K77" s="139" t="n">
-        <v>33</v>
+        <v>41.25</v>
       </c>
       <c r="L77" s="139" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="M77" s="139" t="n">
-        <v>21</v>
+        <v>26.25</v>
       </c>
       <c r="N77" s="139" t="n">
-        <v>33</v>
+        <v>41.25</v>
       </c>
       <c r="O77" s="139" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="P77" s="139" t="n">
-        <v>21</v>
+        <v>26.25</v>
       </c>
       <c r="Q77" s="139" t="n">
-        <v>33</v>
+        <v>41.25</v>
       </c>
       <c r="R77" s="139" t="n">
-        <v>13.5</v>
+        <v>18</v>
       </c>
       <c r="S77" s="139" t="n">
-        <v>13.5</v>
+        <v>18</v>
       </c>
       <c r="T77" s="139" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="U77" s="139" t="n">
-        <v>21</v>
+        <v>26.25</v>
       </c>
       <c r="V77" s="139" t="n">
-        <v>33</v>
+        <v>41.25</v>
       </c>
       <c r="W77" s="139" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="X77" s="139" t="n">
-        <v>21</v>
+        <v>26.25</v>
       </c>
       <c r="Y77" s="139" t="n">
-        <v>33</v>
+        <v>41.25</v>
       </c>
       <c r="Z77" s="139" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="AA77" s="139" t="n">
-        <v>21</v>
+        <v>26.25</v>
       </c>
       <c r="AB77" s="139" t="n">
-        <v>33</v>
+        <v>41.25</v>
       </c>
     </row>
     <row r="78" ht="24" customHeight="1">
@@ -10847,70 +10847,70 @@
       </c>
       <c r="F78" s="123" t="inlineStr"/>
       <c r="G78" s="139" t="n">
-        <v>1.223091976516634</v>
+        <v>1.630789302022179</v>
       </c>
       <c r="H78" s="139" t="n">
-        <v>1.223091976516634</v>
+        <v>1.630789302022179</v>
       </c>
       <c r="I78" s="139" t="n">
-        <v>3.261578604044357</v>
+        <v>4.076973255055447</v>
       </c>
       <c r="J78" s="139" t="n">
-        <v>1.902587519025875</v>
+        <v>2.378234398782344</v>
       </c>
       <c r="K78" s="139" t="n">
-        <v>2.989780387040661</v>
+        <v>3.737225483800826</v>
       </c>
       <c r="L78" s="139" t="n">
-        <v>3.261578604044358</v>
+        <v>4.076973255055448</v>
       </c>
       <c r="M78" s="139" t="n">
-        <v>1.902587519025875</v>
+        <v>2.378234398782344</v>
       </c>
       <c r="N78" s="139" t="n">
-        <v>2.989780387040661</v>
+        <v>3.737225483800827</v>
       </c>
       <c r="O78" s="139" t="n">
-        <v>3.261578604044357</v>
+        <v>4.076973255055447</v>
       </c>
       <c r="P78" s="139" t="n">
-        <v>1.902587519025875</v>
+        <v>2.378234398782344</v>
       </c>
       <c r="Q78" s="139" t="n">
-        <v>2.989780387040661</v>
+        <v>3.737225483800826</v>
       </c>
       <c r="R78" s="139" t="n">
-        <v>0.7690048439773882</v>
+        <v>1.025339791969851</v>
       </c>
       <c r="S78" s="139" t="n">
-        <v>0.7690048439773882</v>
+        <v>1.025339791969851</v>
       </c>
       <c r="T78" s="139" t="n">
-        <v>2.170111239321003</v>
+        <v>2.712639049151254</v>
       </c>
       <c r="U78" s="139" t="n">
-        <v>1.265898222937252</v>
+        <v>1.582372778671565</v>
       </c>
       <c r="V78" s="139" t="n">
-        <v>1.989268636044253</v>
+        <v>2.486585795055316</v>
       </c>
       <c r="W78" s="139" t="n">
-        <v>2.170111239321003</v>
+        <v>2.712639049151254</v>
       </c>
       <c r="X78" s="139" t="n">
-        <v>1.265898222937252</v>
+        <v>1.582372778671564</v>
       </c>
       <c r="Y78" s="139" t="n">
-        <v>1.989268636044253</v>
+        <v>2.486585795055316</v>
       </c>
       <c r="Z78" s="139" t="n">
-        <v>2.170111239321003</v>
+        <v>2.712639049151254</v>
       </c>
       <c r="AA78" s="139" t="n">
-        <v>1.265898222937252</v>
+        <v>1.582372778671565</v>
       </c>
       <c r="AB78" s="139" t="n">
-        <v>1.989268636044253</v>
+        <v>2.486585795055316</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
@@ -11261,70 +11261,70 @@
       </c>
       <c r="F84" s="123" t="inlineStr"/>
       <c r="G84" s="128" t="n">
-        <v>0.4897879746905529</v>
+        <v>0.4895628596114459</v>
       </c>
       <c r="H84" s="128" t="n">
-        <v>0.4914088032601224</v>
+        <v>0.4907784810386232</v>
       </c>
       <c r="I84" s="128" t="n">
-        <v>0.4894048771121579</v>
+        <v>0.489301405072798</v>
       </c>
       <c r="J84" s="128" t="n">
-        <v>0.4897480495016082</v>
+        <v>0.4895759434087582</v>
       </c>
       <c r="K84" s="128" t="n">
-        <v>0.4894271248846355</v>
+        <v>0.4893192030608538</v>
       </c>
       <c r="L84" s="128" t="n">
-        <v>0.4900633295905272</v>
+        <v>0.4898281691724303</v>
       </c>
       <c r="M84" s="128" t="n">
-        <v>0.490843259166844</v>
+        <v>0.4904521150256014</v>
       </c>
       <c r="N84" s="128" t="n">
-        <v>0.4901138968664241</v>
+        <v>0.4898686218055564</v>
       </c>
       <c r="O84" s="128" t="n">
-        <v>0.4899222334971803</v>
+        <v>0.4897152917055201</v>
       </c>
       <c r="P84" s="128" t="n">
-        <v>0.4906085729711289</v>
+        <v>0.4902643649822608</v>
       </c>
       <c r="Q84" s="128" t="n">
-        <v>0.4899667319161581</v>
+        <v>0.4897508895210251</v>
       </c>
       <c r="R84" s="128" t="n">
-        <v>0.4897879746905529</v>
+        <v>0.4895628596114459</v>
       </c>
       <c r="S84" s="128" t="n">
-        <v>0.4914088032601224</v>
+        <v>0.4907784810386232</v>
       </c>
       <c r="T84" s="128" t="n">
-        <v>0.4894048771121579</v>
+        <v>0.489301405072798</v>
       </c>
       <c r="U84" s="128" t="n">
-        <v>0.4897480495016082</v>
+        <v>0.4895759434087582</v>
       </c>
       <c r="V84" s="128" t="n">
-        <v>0.4894271248846355</v>
+        <v>0.4893192030608538</v>
       </c>
       <c r="W84" s="128" t="n">
-        <v>0.4900633295905272</v>
+        <v>0.4898281691724303</v>
       </c>
       <c r="X84" s="128" t="n">
-        <v>0.490843259166844</v>
+        <v>0.4904521150256014</v>
       </c>
       <c r="Y84" s="128" t="n">
-        <v>0.4901138968664241</v>
+        <v>0.4898686218055564</v>
       </c>
       <c r="Z84" s="128" t="n">
-        <v>0.4899222334971803</v>
+        <v>0.4897152917055201</v>
       </c>
       <c r="AA84" s="128" t="n">
-        <v>0.4906085729711289</v>
+        <v>0.4902643649822608</v>
       </c>
       <c r="AB84" s="128" t="n">
-        <v>0.4899667319161581</v>
+        <v>0.4897508895210251</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
@@ -11355,70 +11355,70 @@
       </c>
       <c r="F85" s="123" t="inlineStr"/>
       <c r="G85" s="128" t="n">
-        <v>0.5102120253094471</v>
+        <v>0.5104371403885539</v>
       </c>
       <c r="H85" s="128" t="n">
-        <v>0.5085911967398776</v>
+        <v>0.5092215189613769</v>
       </c>
       <c r="I85" s="128" t="n">
-        <v>0.5105951228878421</v>
+        <v>0.5106985949272019</v>
       </c>
       <c r="J85" s="128" t="n">
-        <v>0.510251950498392</v>
+        <v>0.510424056591242</v>
       </c>
       <c r="K85" s="128" t="n">
-        <v>0.5105728751153646</v>
+        <v>0.5106807969391461</v>
       </c>
       <c r="L85" s="128" t="n">
-        <v>0.5099366704094728</v>
+        <v>0.5101718308275697</v>
       </c>
       <c r="M85" s="128" t="n">
-        <v>0.5091567408331559</v>
+        <v>0.5095478849743985</v>
       </c>
       <c r="N85" s="128" t="n">
-        <v>0.5098861031335759</v>
+        <v>0.5101313781944437</v>
       </c>
       <c r="O85" s="128" t="n">
-        <v>0.5100777665028198</v>
+        <v>0.5102847082944798</v>
       </c>
       <c r="P85" s="128" t="n">
-        <v>0.5093914270288711</v>
+        <v>0.5097356350177393</v>
       </c>
       <c r="Q85" s="128" t="n">
-        <v>0.510033268083842</v>
+        <v>0.510249110478975</v>
       </c>
       <c r="R85" s="128" t="n">
-        <v>0.5102120253094471</v>
+        <v>0.5104371403885539</v>
       </c>
       <c r="S85" s="128" t="n">
-        <v>0.5085911967398776</v>
+        <v>0.5092215189613769</v>
       </c>
       <c r="T85" s="128" t="n">
-        <v>0.5105951228878421</v>
+        <v>0.5106985949272019</v>
       </c>
       <c r="U85" s="128" t="n">
-        <v>0.510251950498392</v>
+        <v>0.510424056591242</v>
       </c>
       <c r="V85" s="128" t="n">
-        <v>0.5105728751153646</v>
+        <v>0.5106807969391461</v>
       </c>
       <c r="W85" s="128" t="n">
-        <v>0.5099366704094728</v>
+        <v>0.5101718308275697</v>
       </c>
       <c r="X85" s="128" t="n">
-        <v>0.5091567408331559</v>
+        <v>0.5095478849743985</v>
       </c>
       <c r="Y85" s="128" t="n">
-        <v>0.5098861031335759</v>
+        <v>0.5101313781944437</v>
       </c>
       <c r="Z85" s="128" t="n">
-        <v>0.5100777665028198</v>
+        <v>0.5102847082944798</v>
       </c>
       <c r="AA85" s="128" t="n">
-        <v>0.5093914270288711</v>
+        <v>0.5097356350177393</v>
       </c>
       <c r="AB85" s="128" t="n">
-        <v>0.510033268083842</v>
+        <v>0.510249110478975</v>
       </c>
     </row>
     <row r="86" ht="24" customHeight="1">
@@ -12225,70 +12225,70 @@
       </c>
       <c r="F94" s="123" t="inlineStr"/>
       <c r="G94" s="126" t="n">
-        <v>119566.4240550489</v>
+        <v>159232.8020736146</v>
       </c>
       <c r="H94" s="126" t="n">
-        <v>43066.9807335277</v>
+        <v>57233.54431158697</v>
       </c>
       <c r="I94" s="126" t="n">
-        <v>227285.8525350946</v>
+        <v>283952.1076094415</v>
       </c>
       <c r="J94" s="126" t="n">
-        <v>132823.6346513869</v>
+        <v>165878.9504827817</v>
       </c>
       <c r="K94" s="126" t="n">
-        <v>208369.8373731809</v>
+        <v>260313.9042087232</v>
       </c>
       <c r="L94" s="126" t="n">
-        <v>100353.4380237983</v>
+        <v>125286.5916543615</v>
       </c>
       <c r="M94" s="126" t="n">
-        <v>58779.72382398446</v>
+        <v>73324.0642851264</v>
       </c>
       <c r="N94" s="126" t="n">
-        <v>92015.12608353581</v>
+        <v>114870.5161924741</v>
       </c>
       <c r="O94" s="126" t="n">
-        <v>113953.3400983082</v>
+        <v>142286.4687796304</v>
       </c>
       <c r="P94" s="126" t="n">
-        <v>66713.00054041948</v>
+        <v>83240.65967997638</v>
       </c>
       <c r="Q94" s="126" t="n">
-        <v>104481.702554051</v>
+        <v>130453.7365458037</v>
       </c>
       <c r="R94" s="126" t="n">
-        <v>119566.4240550489</v>
+        <v>159232.8020736146</v>
       </c>
       <c r="S94" s="126" t="n">
-        <v>43066.9807335277</v>
+        <v>57233.54431158697</v>
       </c>
       <c r="T94" s="126" t="n">
-        <v>227285.8525350946</v>
+        <v>283952.1076094415</v>
       </c>
       <c r="U94" s="126" t="n">
-        <v>132823.6346513869</v>
+        <v>165878.9504827817</v>
       </c>
       <c r="V94" s="126" t="n">
-        <v>208369.8373731809</v>
+        <v>260313.9042087232</v>
       </c>
       <c r="W94" s="126" t="n">
-        <v>100353.4380237983</v>
+        <v>125286.5916543615</v>
       </c>
       <c r="X94" s="126" t="n">
-        <v>58779.72382398446</v>
+        <v>73324.0642851264</v>
       </c>
       <c r="Y94" s="126" t="n">
-        <v>92015.12608353581</v>
+        <v>114870.5161924741</v>
       </c>
       <c r="Z94" s="126" t="n">
-        <v>113953.3400983082</v>
+        <v>142286.4687796304</v>
       </c>
       <c r="AA94" s="126" t="n">
-        <v>66713.00054041948</v>
+        <v>83240.65967997638</v>
       </c>
       <c r="AB94" s="126" t="n">
-        <v>104481.702554051</v>
+        <v>130453.7365458037</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
@@ -12319,70 +12319,70 @@
       </c>
       <c r="F95" s="123" t="inlineStr"/>
       <c r="G95" s="126" t="n">
-        <v>321433.5759449532</v>
+        <v>428767.1979263856</v>
       </c>
       <c r="H95" s="126" t="n">
-        <v>114433.0192664728</v>
+        <v>152766.455688413</v>
       </c>
       <c r="I95" s="126" t="n">
-        <v>612714.1474667725</v>
+        <v>766047.892391463</v>
       </c>
       <c r="J95" s="126" t="n">
-        <v>357176.3653495767</v>
+        <v>446621.0495176552</v>
       </c>
       <c r="K95" s="126" t="n">
-        <v>561630.1626271219</v>
+        <v>702186.0957914591</v>
       </c>
       <c r="L95" s="126" t="n">
-        <v>269246.5619762017</v>
+        <v>336713.4083476944</v>
       </c>
       <c r="M95" s="126" t="n">
-        <v>156820.2761782036</v>
+        <v>196175.9357158656</v>
       </c>
       <c r="N95" s="126" t="n">
-        <v>246784.8739171512</v>
+        <v>308629.4838079407</v>
       </c>
       <c r="O95" s="126" t="n">
-        <v>306046.6599016918</v>
+        <v>382713.5312221787</v>
       </c>
       <c r="P95" s="126" t="n">
-        <v>178286.9994615063</v>
+        <v>223009.3403208967</v>
       </c>
       <c r="Q95" s="126" t="n">
-        <v>280518.2974465535</v>
+        <v>350796.2634545615</v>
       </c>
       <c r="R95" s="126" t="n">
-        <v>321433.5759449532</v>
+        <v>428767.1979263856</v>
       </c>
       <c r="S95" s="126" t="n">
-        <v>114433.0192664728</v>
+        <v>152766.455688413</v>
       </c>
       <c r="T95" s="126" t="n">
-        <v>612714.1474667725</v>
+        <v>766047.892391463</v>
       </c>
       <c r="U95" s="126" t="n">
-        <v>357176.3653495767</v>
+        <v>446621.0495176552</v>
       </c>
       <c r="V95" s="126" t="n">
-        <v>561630.1626271219</v>
+        <v>702186.0957914591</v>
       </c>
       <c r="W95" s="126" t="n">
-        <v>269246.5619762017</v>
+        <v>336713.4083476944</v>
       </c>
       <c r="X95" s="126" t="n">
-        <v>156820.2761782036</v>
+        <v>196175.9357158656</v>
       </c>
       <c r="Y95" s="126" t="n">
-        <v>246784.8739171512</v>
+        <v>308629.4838079407</v>
       </c>
       <c r="Z95" s="126" t="n">
-        <v>306046.6599016918</v>
+        <v>382713.5312221787</v>
       </c>
       <c r="AA95" s="126" t="n">
-        <v>178286.9994615063</v>
+        <v>223009.3403208967</v>
       </c>
       <c r="AB95" s="126" t="n">
-        <v>280518.2974465535</v>
+        <v>350796.2634545615</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
@@ -12413,70 +12413,70 @@
       </c>
       <c r="F96" s="123" t="inlineStr"/>
       <c r="G96" s="126" t="n">
-        <v>441000.0000000021</v>
+        <v>588000.0000000002</v>
       </c>
       <c r="H96" s="126" t="n">
-        <v>157500.0000000005</v>
+        <v>210000</v>
       </c>
       <c r="I96" s="126" t="n">
-        <v>840000.0000018671</v>
+        <v>1050000.000000905</v>
       </c>
       <c r="J96" s="126" t="n">
-        <v>490000.0000009636</v>
+        <v>612500.0000004369</v>
       </c>
       <c r="K96" s="126" t="n">
-        <v>770000.0000003028</v>
+        <v>962500.0000001823</v>
       </c>
       <c r="L96" s="126" t="n">
-        <v>369600</v>
+        <v>462000.0000020558</v>
       </c>
       <c r="M96" s="126" t="n">
-        <v>215600.000002188</v>
+        <v>269500.000000992</v>
       </c>
       <c r="N96" s="126" t="n">
-        <v>338800.000000687</v>
+        <v>423500.0000004148</v>
       </c>
       <c r="O96" s="126" t="n">
-        <v>420000</v>
+        <v>525000.0000018091</v>
       </c>
       <c r="P96" s="126" t="n">
-        <v>245000.0000019257</v>
+        <v>306250.0000008731</v>
       </c>
       <c r="Q96" s="126" t="n">
-        <v>385000.0000006045</v>
+        <v>481250.0000003652</v>
       </c>
       <c r="R96" s="126" t="n">
-        <v>441000.0000000021</v>
+        <v>588000.0000000002</v>
       </c>
       <c r="S96" s="126" t="n">
-        <v>157500.0000000005</v>
+        <v>210000</v>
       </c>
       <c r="T96" s="126" t="n">
-        <v>840000.0000018671</v>
+        <v>1050000.000000905</v>
       </c>
       <c r="U96" s="126" t="n">
-        <v>490000.0000009636</v>
+        <v>612500.0000004369</v>
       </c>
       <c r="V96" s="126" t="n">
-        <v>770000.0000003028</v>
+        <v>962500.0000001823</v>
       </c>
       <c r="W96" s="126" t="n">
-        <v>369600</v>
+        <v>462000.0000020558</v>
       </c>
       <c r="X96" s="126" t="n">
-        <v>215600.000002188</v>
+        <v>269500.000000992</v>
       </c>
       <c r="Y96" s="126" t="n">
-        <v>338800.000000687</v>
+        <v>423500.0000004148</v>
       </c>
       <c r="Z96" s="126" t="n">
-        <v>420000</v>
+        <v>525000.0000018091</v>
       </c>
       <c r="AA96" s="126" t="n">
-        <v>245000.0000019257</v>
+        <v>306250.0000008731</v>
       </c>
       <c r="AB96" s="126" t="n">
-        <v>385000.0000006045</v>
+        <v>481250.0000003652</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
@@ -12507,70 +12507,70 @@
       </c>
       <c r="F97" s="123" t="inlineStr"/>
       <c r="G97" s="126" t="n">
-        <v>189000.000000001</v>
+        <v>252000.0000000002</v>
       </c>
       <c r="H97" s="126" t="n">
-        <v>67500.00000000022</v>
+        <v>90000</v>
       </c>
       <c r="I97" s="126" t="n">
-        <v>360000.0000008002</v>
+        <v>450000.0000003878</v>
       </c>
       <c r="J97" s="126" t="n">
-        <v>210000.000000413</v>
+        <v>262500.0000001873</v>
       </c>
       <c r="K97" s="126" t="n">
-        <v>330000.0000001298</v>
+        <v>412500.0000000783</v>
       </c>
       <c r="L97" s="126" t="n">
-        <v>158400</v>
+        <v>198000.0000008811</v>
       </c>
       <c r="M97" s="126" t="n">
-        <v>92400.00000093774</v>
+        <v>115500.0000004251</v>
       </c>
       <c r="N97" s="126" t="n">
-        <v>145200.0000002945</v>
+        <v>181500.0000001778</v>
       </c>
       <c r="O97" s="126" t="n">
-        <v>180000</v>
+        <v>225000.0000007753</v>
       </c>
       <c r="P97" s="126" t="n">
-        <v>105000.0000008253</v>
+        <v>131250.0000003742</v>
       </c>
       <c r="Q97" s="126" t="n">
-        <v>165000.0000002591</v>
+        <v>206250.0000001566</v>
       </c>
       <c r="R97" s="126" t="n">
-        <v>189000.000000001</v>
+        <v>252000.0000000002</v>
       </c>
       <c r="S97" s="126" t="n">
-        <v>67500.00000000022</v>
+        <v>90000</v>
       </c>
       <c r="T97" s="126" t="n">
-        <v>360000.0000008002</v>
+        <v>450000.0000003878</v>
       </c>
       <c r="U97" s="126" t="n">
-        <v>210000.000000413</v>
+        <v>262500.0000001873</v>
       </c>
       <c r="V97" s="126" t="n">
-        <v>330000.0000001298</v>
+        <v>412500.0000000783</v>
       </c>
       <c r="W97" s="126" t="n">
-        <v>158400</v>
+        <v>198000.0000008811</v>
       </c>
       <c r="X97" s="126" t="n">
-        <v>92400.00000093774</v>
+        <v>115500.0000004251</v>
       </c>
       <c r="Y97" s="126" t="n">
-        <v>145200.0000002945</v>
+        <v>181500.0000001778</v>
       </c>
       <c r="Z97" s="126" t="n">
-        <v>180000</v>
+        <v>225000.0000007753</v>
       </c>
       <c r="AA97" s="126" t="n">
-        <v>105000.0000008253</v>
+        <v>131250.0000003742</v>
       </c>
       <c r="AB97" s="126" t="n">
-        <v>165000.0000002591</v>
+        <v>206250.0000001566</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1">
@@ -12803,28 +12803,28 @@
         <v>0.08400000000000002</v>
       </c>
       <c r="I100" s="141" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08399999999999999</v>
       </c>
       <c r="J100" s="141" t="n">
         <v>0.08400000000000002</v>
       </c>
       <c r="K100" s="141" t="n">
-        <v>0.08400000000000002</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="L100" s="141" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08399999999999999</v>
       </c>
       <c r="M100" s="141" t="n">
         <v>0.08399999999999999</v>
       </c>
       <c r="N100" s="141" t="n">
+        <v>0.08400000000000002</v>
+      </c>
+      <c r="O100" s="141" t="n">
         <v>0.08399999999999999</v>
       </c>
-      <c r="O100" s="141" t="n">
+      <c r="P100" s="141" t="n">
         <v>0.08400000000000002</v>
-      </c>
-      <c r="P100" s="141" t="n">
-        <v>0.08400000000000001</v>
       </c>
       <c r="Q100" s="141" t="n">
         <v>0.08400000000000002</v>
@@ -12836,28 +12836,28 @@
         <v>0.08400000000000002</v>
       </c>
       <c r="T100" s="141" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08399999999999999</v>
       </c>
       <c r="U100" s="141" t="n">
         <v>0.08400000000000002</v>
       </c>
       <c r="V100" s="141" t="n">
-        <v>0.08400000000000002</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="W100" s="141" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08399999999999999</v>
       </c>
       <c r="X100" s="141" t="n">
         <v>0.08399999999999999</v>
       </c>
       <c r="Y100" s="141" t="n">
+        <v>0.08400000000000002</v>
+      </c>
+      <c r="Z100" s="141" t="n">
         <v>0.08399999999999999</v>
       </c>
-      <c r="Z100" s="141" t="n">
+      <c r="AA100" s="141" t="n">
         <v>0.08400000000000002</v>
-      </c>
-      <c r="AA100" s="141" t="n">
-        <v>0.08400000000000001</v>
       </c>
       <c r="AB100" s="141" t="n">
         <v>0.08400000000000002</v>
@@ -12903,7 +12903,7 @@
         <v>0.09800000000000002</v>
       </c>
       <c r="K101" s="141" t="n">
-        <v>0.09800000000000002</v>
+        <v>0.098</v>
       </c>
       <c r="L101" s="141" t="n">
         <v>0.098</v>
@@ -12912,13 +12912,13 @@
         <v>0.098</v>
       </c>
       <c r="N101" s="141" t="n">
+        <v>0.09800000000000002</v>
+      </c>
+      <c r="O101" s="141" t="n">
         <v>0.098</v>
       </c>
-      <c r="O101" s="141" t="n">
+      <c r="P101" s="141" t="n">
         <v>0.09800000000000002</v>
-      </c>
-      <c r="P101" s="141" t="n">
-        <v>0.098</v>
       </c>
       <c r="Q101" s="141" t="n">
         <v>0.09800000000000002</v>
@@ -12936,7 +12936,7 @@
         <v>0.09800000000000002</v>
       </c>
       <c r="V101" s="141" t="n">
-        <v>0.09800000000000002</v>
+        <v>0.098</v>
       </c>
       <c r="W101" s="141" t="n">
         <v>0.098</v>
@@ -12945,13 +12945,13 @@
         <v>0.098</v>
       </c>
       <c r="Y101" s="141" t="n">
+        <v>0.09800000000000002</v>
+      </c>
+      <c r="Z101" s="141" t="n">
         <v>0.098</v>
       </c>
-      <c r="Z101" s="141" t="n">
+      <c r="AA101" s="141" t="n">
         <v>0.09800000000000002</v>
-      </c>
-      <c r="AA101" s="141" t="n">
-        <v>0.098</v>
       </c>
       <c r="AB101" s="141" t="n">
         <v>0.09800000000000002</v>
@@ -16357,70 +16357,70 @@
         </is>
       </c>
       <c r="G144" s="145" t="n">
-        <v>1.71709536116388</v>
+        <v>2.12354528738614</v>
       </c>
       <c r="H144" s="145" t="n">
-        <v>1.63932447237903</v>
+        <v>2.045774398601298</v>
       </c>
       <c r="I144" s="146" t="n">
-        <v>3.840973312069803</v>
+        <v>4.696214229179318</v>
       </c>
       <c r="J144" s="146" t="n">
-        <v>2.437790821299018</v>
+        <v>2.923807338058453</v>
       </c>
       <c r="K144" s="146" t="n">
-        <v>3.67523902935652</v>
+        <v>4.445550738342776</v>
       </c>
       <c r="L144" s="146" t="n">
-        <v>3.84091807921999</v>
+        <v>4.696158996035751</v>
       </c>
       <c r="M144" s="146" t="n">
-        <v>2.437737965759786</v>
+        <v>2.923754482170276</v>
       </c>
       <c r="N144" s="146" t="n">
-        <v>3.675187653863974</v>
+        <v>4.44549936268872</v>
       </c>
       <c r="O144" s="146" t="n">
-        <v>3.840929914725353</v>
+        <v>4.696170831625423</v>
       </c>
       <c r="P144" s="146" t="n">
-        <v>2.437749291834332</v>
+        <v>2.923765808342443</v>
       </c>
       <c r="Q144" s="146" t="n">
-        <v>3.675198662845537</v>
+        <v>4.44551037171547</v>
       </c>
       <c r="R144" s="145" t="n">
-        <v>1.09260513458614</v>
+        <v>1.348155794798428</v>
       </c>
       <c r="S144" s="145" t="n">
-        <v>1.09257346731619</v>
+        <v>1.348124127528474</v>
       </c>
       <c r="T144" s="146" t="n">
-        <v>2.611380326955709</v>
+        <v>3.180420093234884</v>
       </c>
       <c r="U144" s="146" t="n">
-        <v>1.734658316379735</v>
+        <v>2.058032373410724</v>
       </c>
       <c r="V144" s="146" t="n">
-        <v>2.542071709751747</v>
+        <v>3.054603308830421</v>
       </c>
       <c r="W144" s="146" t="n">
-        <v>2.611343577441835</v>
+        <v>3.18038334352556</v>
       </c>
       <c r="X144" s="146" t="n">
-        <v>1.734623148623972</v>
+        <v>2.057997205422789</v>
       </c>
       <c r="Y144" s="146" t="n">
-        <v>2.542037526754084</v>
+        <v>3.054569125725295</v>
       </c>
       <c r="Z144" s="146" t="n">
-        <v>2.611351452267597</v>
+        <v>3.180391218407416</v>
       </c>
       <c r="AA144" s="146" t="n">
-        <v>1.734630684496829</v>
+        <v>2.058004741360597</v>
       </c>
       <c r="AB144" s="146" t="n">
-        <v>2.542044851647188</v>
+        <v>3.054576450648465</v>
       </c>
     </row>
     <row r="145" ht="24" customHeight="1">
@@ -16451,70 +16451,70 @@
       </c>
       <c r="F145" s="123" t="inlineStr"/>
       <c r="G145" s="147" t="n">
-        <v>0.02736145326604436</v>
+        <v>0.03383812364373351</v>
       </c>
       <c r="H145" s="147" t="n">
-        <v>0.02612219504715135</v>
+        <v>0.03259886542484061</v>
       </c>
       <c r="I145" s="147" t="n">
-        <v>0.06120487781359238</v>
+        <v>0.07483291205907511</v>
       </c>
       <c r="J145" s="147" t="n">
-        <v>0.03884554180156508</v>
+        <v>0.04659008442313808</v>
       </c>
       <c r="K145" s="147" t="n">
-        <v>0.05856394654465741</v>
+        <v>0.07083865667574059</v>
       </c>
       <c r="L145" s="147" t="n">
-        <v>0.06120399769296943</v>
+        <v>0.07483203193377129</v>
       </c>
       <c r="M145" s="147" t="n">
-        <v>0.03884469956274756</v>
+        <v>0.04658924217876021</v>
       </c>
       <c r="N145" s="147" t="n">
-        <v>0.0585631278899862</v>
+        <v>0.07083783801849576</v>
       </c>
       <c r="O145" s="147" t="n">
-        <v>0.06120418628856768</v>
+        <v>0.07483222053071296</v>
       </c>
       <c r="P145" s="147" t="n">
-        <v>0.0388448800407026</v>
+        <v>0.0465894226582708</v>
       </c>
       <c r="Q145" s="147" t="n">
-        <v>0.05856330331514974</v>
+        <v>0.07083801344437934</v>
       </c>
       <c r="R145" s="147" t="n">
-        <v>0.01741036928080407</v>
+        <v>0.02148250039515629</v>
       </c>
       <c r="S145" s="147" t="n">
-        <v>0.01740986467136513</v>
+        <v>0.02148199578571728</v>
       </c>
       <c r="T145" s="147" t="n">
-        <v>0.04161164393772244</v>
+        <v>0.05067913973540194</v>
       </c>
       <c r="U145" s="147" t="n">
-        <v>0.027641314238953</v>
+        <v>0.03279419296020659</v>
       </c>
       <c r="V145" s="147" t="n">
-        <v>0.04050722974300063</v>
+        <v>0.04867428307780006</v>
       </c>
       <c r="W145" s="147" t="n">
-        <v>0.04161105834409196</v>
+        <v>0.05067855413865702</v>
       </c>
       <c r="X145" s="147" t="n">
-        <v>0.02764075385021308</v>
+        <v>0.03279363256776704</v>
       </c>
       <c r="Y145" s="147" t="n">
-        <v>0.04050668504611645</v>
+        <v>0.04867373837920351</v>
       </c>
       <c r="Z145" s="147" t="n">
-        <v>0.04161118382732482</v>
+        <v>0.05067867962278373</v>
       </c>
       <c r="AA145" s="147" t="n">
-        <v>0.02764087393232247</v>
+        <v>0.03279375265091142</v>
       </c>
       <c r="AB145" s="147" t="n">
-        <v>0.04050680176632016</v>
+        <v>0.04867385509988631</v>
       </c>
     </row>
     <row r="146" ht="15" customHeight="1">
@@ -16545,10 +16545,10 @@
       </c>
       <c r="F146" s="123" t="inlineStr"/>
       <c r="G146" s="148" t="n">
-        <v>0.1400000000000007</v>
+        <v>0.14</v>
       </c>
       <c r="H146" s="148" t="n">
-        <v>0.1399999999999994</v>
+        <v>0.1400000000000002</v>
       </c>
       <c r="I146" s="148" t="n">
         <v>0.1400000000000002</v>
@@ -16557,58 +16557,58 @@
         <v>0.1400000000000001</v>
       </c>
       <c r="K146" s="148" t="n">
-        <v>0.1400000000000002</v>
+        <v>0.14</v>
       </c>
       <c r="L146" s="148" t="n">
         <v>0.1400000000000001</v>
       </c>
       <c r="M146" s="148" t="n">
-        <v>0.1400000000000002</v>
+        <v>0.1400000000000001</v>
       </c>
       <c r="N146" s="148" t="n">
         <v>0.1400000000000001</v>
       </c>
       <c r="O146" s="148" t="n">
-        <v>0.14</v>
+        <v>0.1400000000000002</v>
       </c>
       <c r="P146" s="148" t="n">
         <v>0.14</v>
       </c>
       <c r="Q146" s="148" t="n">
+        <v>0.1400000000000001</v>
+      </c>
+      <c r="R146" s="148" t="n">
         <v>0.1400000000000002</v>
       </c>
-      <c r="R146" s="148" t="n">
-        <v>0.1399999999999984</v>
-      </c>
       <c r="S146" s="148" t="n">
-        <v>0.1400000000000003</v>
+        <v>0.1400000000000001</v>
       </c>
       <c r="T146" s="148" t="n">
-        <v>0.1400000000000001</v>
+        <v>0.1400000000000002</v>
       </c>
       <c r="U146" s="148" t="n">
-        <v>0.1400000000000001</v>
+        <v>0.1400000000000002</v>
       </c>
       <c r="V146" s="148" t="n">
-        <v>0.1400000000000002</v>
+        <v>0.14</v>
       </c>
       <c r="W146" s="148" t="n">
-        <v>0.1400000000000001</v>
+        <v>0.14</v>
       </c>
       <c r="X146" s="148" t="n">
         <v>0.1400000000000002</v>
       </c>
       <c r="Y146" s="148" t="n">
-        <v>0.1400000000000002</v>
+        <v>0.14</v>
       </c>
       <c r="Z146" s="148" t="n">
-        <v>0.1400000000000002</v>
+        <v>0.1400000000000001</v>
       </c>
       <c r="AA146" s="148" t="n">
-        <v>0.1400000000000002</v>
+        <v>0.14</v>
       </c>
       <c r="AB146" s="148" t="n">
-        <v>0.1400000000000002</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="147" ht="15" customHeight="1">
@@ -16639,70 +16639,70 @@
       </c>
       <c r="F147" s="123" t="inlineStr"/>
       <c r="G147" s="149" t="n">
-        <v>9.294465971293588</v>
+        <v>9.304655023369707</v>
       </c>
       <c r="H147" s="149" t="n">
-        <v>9.301157128290461</v>
+        <v>9.309661987010314</v>
       </c>
       <c r="I147" s="149" t="n">
-        <v>8.26053907119373</v>
+        <v>8.263155178732774</v>
       </c>
       <c r="J147" s="149" t="n">
-        <v>8.779169047304672</v>
+        <v>8.78464917363274</v>
       </c>
       <c r="K147" s="149" t="n">
-        <v>8.603345435319053</v>
+        <v>8.607543752935813</v>
       </c>
       <c r="L147" s="149" t="n">
-        <v>8.260508913610217</v>
+        <v>8.263131103550545</v>
       </c>
       <c r="M147" s="149" t="n">
-        <v>8.779140022290076</v>
+        <v>8.78462613791806</v>
       </c>
       <c r="N147" s="149" t="n">
-        <v>8.603322091946325</v>
+        <v>8.607525165824706</v>
       </c>
       <c r="O147" s="149" t="n">
-        <v>8.260515375934466</v>
+        <v>8.2631362625084</v>
       </c>
       <c r="P147" s="149" t="n">
-        <v>8.779146241906512</v>
+        <v>8.784631074122894</v>
       </c>
       <c r="Q147" s="149" t="n">
-        <v>8.603327094125458</v>
+        <v>8.607529148794638</v>
       </c>
       <c r="R147" s="149" t="n">
-        <v>9.293795914398222</v>
+        <v>9.304150354362317</v>
       </c>
       <c r="S147" s="149" t="n">
-        <v>9.293826941530417</v>
+        <v>9.304174178363924</v>
       </c>
       <c r="T147" s="149" t="n">
-        <v>8.258234879241172</v>
+        <v>8.261312312569641</v>
       </c>
       <c r="U147" s="149" t="n">
-        <v>8.770015273563908</v>
+        <v>8.777332206387689</v>
       </c>
       <c r="V147" s="149" t="n">
-        <v>8.598470406859159</v>
+        <v>8.603646026475925</v>
       </c>
       <c r="W147" s="149" t="n">
-        <v>8.258204667761646</v>
+        <v>8.261288202912015</v>
       </c>
       <c r="X147" s="149" t="n">
-        <v>8.769985865096366</v>
+        <v>8.777308925661583</v>
       </c>
       <c r="Y147" s="149" t="n">
-        <v>8.598446937988006</v>
+        <v>8.603627359138521</v>
       </c>
       <c r="Z147" s="149" t="n">
-        <v>8.258211141635186</v>
+        <v>8.26129336925753</v>
       </c>
       <c r="AA147" s="149" t="n">
-        <v>8.76999216688346</v>
+        <v>8.777313914369975</v>
       </c>
       <c r="AB147" s="149" t="n">
-        <v>8.598451967060122</v>
+        <v>8.603631359300039</v>
       </c>
     </row>
     <row r="148" ht="15" customHeight="1">
@@ -16733,70 +16733,70 @@
       </c>
       <c r="F148" s="123" t="inlineStr"/>
       <c r="G148" s="149" t="n">
-        <v>7.945131357462766</v>
+        <v>7.949483895568179</v>
       </c>
       <c r="H148" s="149" t="n">
-        <v>7.948802369923402</v>
+        <v>7.952236738937815</v>
       </c>
       <c r="I148" s="149" t="n">
-        <v>7.589419494649696</v>
+        <v>7.590447831606477</v>
       </c>
       <c r="J148" s="149" t="n">
-        <v>7.771672791417888</v>
+        <v>7.773829045586591</v>
       </c>
       <c r="K148" s="149" t="n">
-        <v>7.711424795595276</v>
+        <v>7.713095356621857</v>
       </c>
       <c r="L148" s="149" t="n">
-        <v>7.589674281009808</v>
+        <v>7.590651679602107</v>
       </c>
       <c r="M148" s="149" t="n">
-        <v>7.772117993610947</v>
+        <v>7.774185272714031</v>
       </c>
       <c r="N148" s="149" t="n">
-        <v>7.711699345282875</v>
+        <v>7.713315027363903</v>
       </c>
       <c r="O148" s="149" t="n">
-        <v>7.589619682930309</v>
+        <v>7.590607997247229</v>
       </c>
       <c r="P148" s="149" t="n">
-        <v>7.772022589828367</v>
+        <v>7.774108936209268</v>
       </c>
       <c r="Q148" s="149" t="n">
-        <v>7.711640511887304</v>
+        <v>7.713267954217387</v>
       </c>
       <c r="R148" s="149" t="n">
-        <v>7.945059764526371</v>
+        <v>7.949429724025213</v>
       </c>
       <c r="S148" s="149" t="n">
-        <v>7.945761329735673</v>
+        <v>7.949956107134365</v>
       </c>
       <c r="T148" s="149" t="n">
-        <v>7.58849720586591</v>
+        <v>7.589710011097772</v>
       </c>
       <c r="U148" s="149" t="n">
-        <v>7.767982845896669</v>
+        <v>7.770877413497884</v>
       </c>
       <c r="V148" s="149" t="n">
-        <v>7.709459418046734</v>
+        <v>7.711523175013582</v>
       </c>
       <c r="W148" s="149" t="n">
-        <v>7.588751961630682</v>
+        <v>7.589913839513043</v>
       </c>
       <c r="X148" s="149" t="n">
-        <v>7.768427883730142</v>
+        <v>7.771233535460249</v>
       </c>
       <c r="Y148" s="149" t="n">
-        <v>7.709733911168515</v>
+        <v>7.711742809559393</v>
       </c>
       <c r="Z148" s="149" t="n">
-        <v>7.588697370107456</v>
+        <v>7.589870161354023</v>
       </c>
       <c r="AA148" s="149" t="n">
-        <v>7.768332515168451</v>
+        <v>7.771157221491362</v>
       </c>
       <c r="AB148" s="149" t="n">
-        <v>7.709675089894425</v>
+        <v>7.711695744169331</v>
       </c>
     </row>
     <row r="149" ht="24" customHeight="1">
@@ -16827,70 +16827,70 @@
       </c>
       <c r="F149" s="123" t="inlineStr"/>
       <c r="G149" s="147" t="n">
-        <v>0.02550868504155448</v>
+        <v>0.03136446444908701</v>
       </c>
       <c r="H149" s="147" t="n">
-        <v>0.02426388904929457</v>
+        <v>0.03011966845682712</v>
       </c>
       <c r="I149" s="147" t="n">
-        <v>0.05187676437249567</v>
+        <v>0.06317071078409252</v>
       </c>
       <c r="J149" s="147" t="n">
-        <v>0.03444739418441105</v>
+        <v>0.04108978039149466</v>
       </c>
       <c r="K149" s="147" t="n">
-        <v>0.05081112274515391</v>
+        <v>0.06114398880759384</v>
       </c>
       <c r="L149" s="147" t="n">
-        <v>0.05187546974319215</v>
+        <v>0.06316941615502715</v>
       </c>
       <c r="M149" s="147" t="n">
-        <v>0.03444556044704591</v>
+        <v>0.04108794665395479</v>
       </c>
       <c r="N149" s="147" t="n">
-        <v>0.05080983529091389</v>
+        <v>0.06114270135330013</v>
       </c>
       <c r="O149" s="147" t="n">
-        <v>0.05187574716371444</v>
+        <v>0.06316969357551092</v>
       </c>
       <c r="P149" s="147" t="n">
-        <v>0.03444595339073448</v>
+        <v>0.04108833959769228</v>
       </c>
       <c r="Q149" s="147" t="n">
-        <v>0.05081011117395205</v>
+        <v>0.06114297723635339</v>
       </c>
       <c r="R149" s="147" t="n">
-        <v>0.01624341879946173</v>
+        <v>0.01992517194322811</v>
       </c>
       <c r="S149" s="147" t="n">
-        <v>0.01624121794704754</v>
+        <v>0.01992297109081393</v>
       </c>
       <c r="T149" s="147" t="n">
-        <v>0.03540489373627916</v>
+        <v>0.04291938994179882</v>
       </c>
       <c r="U149" s="147" t="n">
-        <v>0.02471682581843091</v>
+        <v>0.02913637803956356</v>
       </c>
       <c r="V149" s="147" t="n">
-        <v>0.03535010494402219</v>
+        <v>0.04222514047089693</v>
       </c>
       <c r="W149" s="147" t="n">
-        <v>0.03540403234676708</v>
+        <v>0.0429185285524452</v>
       </c>
       <c r="X149" s="147" t="n">
-        <v>0.02471560573007825</v>
+        <v>0.02913515795109464</v>
       </c>
       <c r="Y149" s="147" t="n">
-        <v>0.03534924832848243</v>
+        <v>0.04222428385532143</v>
       </c>
       <c r="Z149" s="147" t="n">
-        <v>0.03540421693020552</v>
+        <v>0.042918713135858</v>
       </c>
       <c r="AA149" s="147" t="n">
-        <v>0.02471586717756076</v>
+        <v>0.02913541939860969</v>
       </c>
       <c r="AB149" s="147" t="n">
-        <v>0.03534943188894641</v>
+        <v>0.04222446741579546</v>
       </c>
     </row>
     <row r="150" ht="24" customHeight="1">
@@ -16921,70 +16921,70 @@
       </c>
       <c r="F150" s="123" t="inlineStr"/>
       <c r="G150" s="150" t="n">
-        <v>1.875832822406664e-12</v>
+        <v>0</v>
       </c>
       <c r="H150" s="150" t="n">
         <v>0</v>
       </c>
       <c r="I150" s="150" t="n">
-        <v>2.667547960299999e-09</v>
+        <v>1.292619344894774e-09</v>
       </c>
       <c r="J150" s="150" t="n">
-        <v>1.37674760480877e-09</v>
+        <v>6.240270522539504e-10</v>
       </c>
       <c r="K150" s="150" t="n">
-        <v>4.326921043684706e-10</v>
+        <v>2.607976057333872e-10</v>
       </c>
       <c r="L150" s="150" t="n">
-        <v>0</v>
+        <v>6.67478161631152e-09</v>
       </c>
       <c r="M150" s="150" t="n">
-        <v>7.103949428710621e-09</v>
+        <v>3.220748112653382e-09</v>
       </c>
       <c r="N150" s="150" t="n">
-        <v>2.23076312977355e-09</v>
+        <v>1.346961653325707e-09</v>
       </c>
       <c r="O150" s="150" t="n">
-        <v>0</v>
+        <v>5.168885763850994e-09</v>
       </c>
       <c r="P150" s="150" t="n">
-        <v>5.502101885213051e-09</v>
+        <v>2.494516593287699e-09</v>
       </c>
       <c r="Q150" s="150" t="n">
-        <v>1.727130438666791e-09</v>
+        <v>1.043645170284435e-09</v>
       </c>
       <c r="R150" s="150" t="n">
-        <v>1.875832822406664e-12</v>
+        <v>0</v>
       </c>
       <c r="S150" s="150" t="n">
         <v>0</v>
       </c>
       <c r="T150" s="150" t="n">
-        <v>2.667547960299999e-09</v>
+        <v>1.292619344894774e-09</v>
       </c>
       <c r="U150" s="150" t="n">
-        <v>1.37674760480877e-09</v>
+        <v>6.240270522539504e-10</v>
       </c>
       <c r="V150" s="150" t="n">
-        <v>4.326921043684706e-10</v>
+        <v>2.607976057333872e-10</v>
       </c>
       <c r="W150" s="150" t="n">
-        <v>0</v>
+        <v>6.67478161631152e-09</v>
       </c>
       <c r="X150" s="150" t="n">
-        <v>7.103949428710621e-09</v>
+        <v>3.220748112653382e-09</v>
       </c>
       <c r="Y150" s="150" t="n">
-        <v>2.23076312977355e-09</v>
+        <v>1.346961653325707e-09</v>
       </c>
       <c r="Z150" s="150" t="n">
-        <v>0</v>
+        <v>5.168885763850994e-09</v>
       </c>
       <c r="AA150" s="150" t="n">
-        <v>5.502101885213051e-09</v>
+        <v>2.494516593287699e-09</v>
       </c>
       <c r="AB150" s="150" t="n">
-        <v>1.727130438666791e-09</v>
+        <v>1.043645170284435e-09</v>
       </c>
     </row>
     <row r="152">
@@ -17049,70 +17049,70 @@
       </c>
       <c r="F153" s="123" t="inlineStr"/>
       <c r="G153" s="150" t="n">
-        <v>1.113210815556326</v>
+        <v>1.486830198990387</v>
       </c>
       <c r="H153" s="150" t="n">
-        <v>1.114523660438694</v>
+        <v>1.488143043872764</v>
       </c>
       <c r="I153" s="151" t="n">
-        <v>3.153855737078547</v>
+        <v>3.94390173844531</v>
       </c>
       <c r="J153" s="151" t="n">
-        <v>1.784194928369909</v>
+        <v>2.23213977590294</v>
       </c>
       <c r="K153" s="151" t="n">
-        <v>2.831870076237649</v>
+        <v>3.542161243792975</v>
       </c>
       <c r="L153" s="151" t="n">
-        <v>3.153836591657454</v>
+        <v>3.943882592731354</v>
       </c>
       <c r="M153" s="151" t="n">
-        <v>1.784178234915861</v>
+        <v>2.232123082103706</v>
       </c>
       <c r="N153" s="151" t="n">
-        <v>2.831854894884217</v>
+        <v>3.542146062279643</v>
       </c>
       <c r="O153" s="151" t="n">
-        <v>3.153840694143365</v>
+        <v>3.94388669530116</v>
       </c>
       <c r="P153" s="151" t="n">
-        <v>1.784181811973243</v>
+        <v>2.232126659257657</v>
       </c>
       <c r="Q153" s="151" t="n">
-        <v>2.831858147979329</v>
+        <v>3.54214931541949</v>
       </c>
       <c r="R153" s="150" t="n">
-        <v>0.700014289580048</v>
+        <v>0.9349231281474634</v>
       </c>
       <c r="S153" s="150" t="n">
-        <v>0.700005694569188</v>
+        <v>0.9349145331365989</v>
       </c>
       <c r="T153" s="151" t="n">
-        <v>2.097771885348189</v>
+        <v>2.623433816359344</v>
       </c>
       <c r="U153" s="151" t="n">
-        <v>1.185488649618506</v>
+        <v>1.483531489065016</v>
       </c>
       <c r="V153" s="151" t="n">
-        <v>1.882837601322518</v>
+        <v>2.355434166676148</v>
       </c>
       <c r="W153" s="151" t="n">
-        <v>2.097759146825363</v>
+        <v>2.62342107764166</v>
       </c>
       <c r="X153" s="151" t="n">
-        <v>1.185477542526925</v>
+        <v>1.483520381743764</v>
       </c>
       <c r="Y153" s="151" t="n">
-        <v>1.882827500316316</v>
+        <v>2.355424065563553</v>
       </c>
       <c r="Z153" s="151" t="n">
-        <v>2.097761876439413</v>
+        <v>2.623423807311532</v>
       </c>
       <c r="AA153" s="151" t="n">
-        <v>1.185479922543897</v>
+        <v>1.483522761824987</v>
       </c>
       <c r="AB153" s="151" t="n">
-        <v>1.882829664783011</v>
+        <v>2.355426230060016</v>
       </c>
     </row>
     <row r="154" ht="15" customHeight="1">
@@ -17143,70 +17143,70 @@
       </c>
       <c r="F154" s="123" t="inlineStr"/>
       <c r="G154" s="150" t="n">
-        <v>0.04248573913293401</v>
+        <v>0.04777779558966159</v>
       </c>
       <c r="H154" s="150" t="n">
-        <v>0.03800360248121382</v>
+        <v>0.04329565893794141</v>
       </c>
       <c r="I154" s="151" t="n">
-        <v>0.06085164375219657</v>
+        <v>0.07052284750191348</v>
       </c>
       <c r="J154" s="151" t="n">
-        <v>0.04962773710894557</v>
+        <v>0.05544216248294227</v>
       </c>
       <c r="K154" s="151" t="n">
-        <v>0.06917736992517988</v>
+        <v>0.07844986359632908</v>
       </c>
       <c r="L154" s="151" t="n">
-        <v>0.06080210844138251</v>
+        <v>0.07047331219180548</v>
       </c>
       <c r="M154" s="151" t="n">
-        <v>0.04957810000815011</v>
+        <v>0.05539252538226503</v>
       </c>
       <c r="N154" s="151" t="n">
-        <v>0.06912768448910267</v>
+        <v>0.07840017816032213</v>
       </c>
       <c r="O154" s="151" t="n">
-        <v>0.06081272315097044</v>
+        <v>0.07048392690121993</v>
       </c>
       <c r="P154" s="151" t="n">
-        <v>0.04958873652980943</v>
+        <v>0.05540316190389129</v>
       </c>
       <c r="Q154" s="151" t="n">
-        <v>0.06913833136828895</v>
+        <v>0.07841082503948879</v>
       </c>
       <c r="R154" s="150" t="n">
-        <v>0.02680534643415587</v>
+        <v>0.03013266533409306</v>
       </c>
       <c r="S154" s="150" t="n">
-        <v>0.02677369187463278</v>
+        <v>0.03010101077456997</v>
       </c>
       <c r="T154" s="151" t="n">
-        <v>0.04308338807996767</v>
+        <v>0.04951818254697807</v>
       </c>
       <c r="U154" s="151" t="n">
-        <v>0.03885971245045097</v>
+        <v>0.04272837587578042</v>
       </c>
       <c r="V154" s="151" t="n">
-        <v>0.05095879864154527</v>
+        <v>0.05712830892326653</v>
       </c>
       <c r="W154" s="151" t="n">
-        <v>0.04305042945845613</v>
+        <v>0.04948522392593631</v>
       </c>
       <c r="X154" s="151" t="n">
-        <v>0.03882668610235376</v>
+        <v>0.04269534952776186</v>
       </c>
       <c r="Y154" s="151" t="n">
-        <v>0.05092574013327326</v>
+        <v>0.05709525041504129</v>
       </c>
       <c r="Z154" s="151" t="n">
-        <v>0.04305749202029362</v>
+        <v>0.04949228648765837</v>
       </c>
       <c r="AA154" s="151" t="n">
-        <v>0.03883376317698627</v>
+        <v>0.04270242660237237</v>
       </c>
       <c r="AB154" s="151" t="n">
-        <v>0.05093282409934952</v>
+        <v>0.05710233438110449</v>
       </c>
     </row>
     <row r="155" ht="15" customHeight="1">
@@ -17331,70 +17331,70 @@
       </c>
       <c r="F156" s="123" t="inlineStr"/>
       <c r="G156" s="150" t="n">
-        <v>0.1083414537470186</v>
+        <v>0.1328416046460465</v>
       </c>
       <c r="H156" s="150" t="n">
-        <v>0.107633003568228</v>
+        <v>0.1321331544672561</v>
       </c>
       <c r="I156" s="151" t="n">
-        <v>0.2339831193583159</v>
+        <v>0.2839542902423469</v>
       </c>
       <c r="J156" s="151" t="n">
-        <v>0.1504877984741485</v>
+        <v>0.1794067985308676</v>
       </c>
       <c r="K156" s="151" t="n">
-        <v>0.2174797461027427</v>
+        <v>0.2629041647027586</v>
       </c>
       <c r="L156" s="151" t="n">
-        <v>0.2340260628416754</v>
+        <v>0.2839972337237082</v>
       </c>
       <c r="M156" s="151" t="n">
-        <v>0.1505308275318445</v>
+        <v>0.1794498275846172</v>
       </c>
       <c r="N156" s="151" t="n">
-        <v>0.2175228191925891</v>
+        <v>0.2629472377908854</v>
       </c>
       <c r="O156" s="151" t="n">
-        <v>0.2340168606654816</v>
+        <v>0.2839880315481977</v>
       </c>
       <c r="P156" s="151" t="n">
-        <v>0.1505216070182965</v>
+        <v>0.1794406070721735</v>
       </c>
       <c r="Q156" s="151" t="n">
-        <v>0.2175135892442209</v>
+        <v>0.2629380078429988</v>
       </c>
       <c r="R156" s="150" t="n">
-        <v>0.07938208693776358</v>
+        <v>0.09478627164445091</v>
       </c>
       <c r="S156" s="150" t="n">
-        <v>0.07940951372560666</v>
+        <v>0.09481369843229404</v>
       </c>
       <c r="T156" s="151" t="n">
-        <v>0.1662610335270309</v>
+        <v>0.199509657197482</v>
       </c>
       <c r="U156" s="151" t="n">
-        <v>0.1112574539563226</v>
+        <v>0.1304988872227758</v>
       </c>
       <c r="V156" s="151" t="n">
-        <v>0.1556768036022249</v>
+        <v>0.185900217878147</v>
       </c>
       <c r="W156" s="151" t="n">
-        <v>0.166289606235896</v>
+        <v>0.1995382299050175</v>
       </c>
       <c r="X156" s="151" t="n">
-        <v>0.1112860836025951</v>
+        <v>0.1305275168664224</v>
       </c>
       <c r="Y156" s="151" t="n">
-        <v>0.1557054625455575</v>
+        <v>0.1859288768203355</v>
       </c>
       <c r="Z156" s="151" t="n">
-        <v>0.1662834835117771</v>
+        <v>0.1995321071813534</v>
       </c>
       <c r="AA156" s="151" t="n">
-        <v>0.1112799486776057</v>
+        <v>0.1305213819421677</v>
       </c>
       <c r="AB156" s="151" t="n">
-        <v>0.1556993213430528</v>
+        <v>0.1859227356181512</v>
       </c>
     </row>
     <row r="157" ht="15" customHeight="1">
@@ -17425,70 +17425,70 @@
       </c>
       <c r="F157" s="123" t="inlineStr"/>
       <c r="G157" s="152" t="n">
-        <v>1.264038008436278</v>
+        <v>1.667449599226095</v>
       </c>
       <c r="H157" s="152" t="n">
-        <v>1.260160266488136</v>
+        <v>1.663571857277961</v>
       </c>
       <c r="I157" s="153" t="n">
-        <v>3.448690500189059</v>
+        <v>4.29837887618957</v>
       </c>
       <c r="J157" s="153" t="n">
-        <v>1.984310463953003</v>
+        <v>2.46698873691675</v>
       </c>
       <c r="K157" s="153" t="n">
-        <v>3.118527192265571</v>
+        <v>3.883515272092063</v>
       </c>
       <c r="L157" s="153" t="n">
-        <v>3.448664762940512</v>
+        <v>4.298353138646868</v>
       </c>
       <c r="M157" s="153" t="n">
-        <v>1.984287162455855</v>
+        <v>2.466965435070589</v>
       </c>
       <c r="N157" s="153" t="n">
-        <v>3.118505398565909</v>
+        <v>3.883493478230851</v>
       </c>
       <c r="O157" s="153" t="n">
-        <v>3.448670277959817</v>
+        <v>4.298358653750578</v>
       </c>
       <c r="P157" s="153" t="n">
-        <v>1.984292155521349</v>
+        <v>2.466970428233721</v>
       </c>
       <c r="Q157" s="153" t="n">
-        <v>3.118510068591839</v>
+        <v>3.883498148301978</v>
       </c>
       <c r="R157" s="152" t="n">
-        <v>0.8062017229519675</v>
+        <v>1.059842065126007</v>
       </c>
       <c r="S157" s="152" t="n">
-        <v>0.8061889001694275</v>
+        <v>1.059829242343463</v>
       </c>
       <c r="T157" s="153" t="n">
-        <v>2.307116306955187</v>
+        <v>2.872461656103805</v>
       </c>
       <c r="U157" s="153" t="n">
-        <v>1.33560581602528</v>
+        <v>1.656758752163572</v>
       </c>
       <c r="V157" s="153" t="n">
-        <v>2.089473203566288</v>
+        <v>2.598462693477561</v>
       </c>
       <c r="W157" s="153" t="n">
-        <v>2.307099182519715</v>
+        <v>2.872444531472614</v>
       </c>
       <c r="X157" s="153" t="n">
-        <v>1.335590312231874</v>
+        <v>1.656743248137948</v>
       </c>
       <c r="Y157" s="153" t="n">
-        <v>2.089458702995147</v>
+        <v>2.59844819279893</v>
       </c>
       <c r="Z157" s="153" t="n">
-        <v>2.307102851971484</v>
+        <v>2.872448200980544</v>
       </c>
       <c r="AA157" s="153" t="n">
-        <v>1.335593634398488</v>
+        <v>1.656746570369527</v>
       </c>
       <c r="AB157" s="153" t="n">
-        <v>2.089461810225414</v>
+        <v>2.598451300059271</v>
       </c>
     </row>
     <row r="158" ht="15" customHeight="1">
@@ -17613,70 +17613,70 @@
       </c>
       <c r="F159" s="123" t="inlineStr"/>
       <c r="G159" s="150" t="n">
-        <v>0.2122220862959302</v>
+        <v>0.215260421728373</v>
       </c>
       <c r="H159" s="150" t="n">
-        <v>0.1383289394592217</v>
+        <v>0.1413672748916645</v>
       </c>
       <c r="I159" s="151" t="n">
-        <v>0.1514475454490726</v>
+        <v>0.1570000865580744</v>
       </c>
       <c r="J159" s="151" t="n">
-        <v>0.3041660054372468</v>
+        <v>0.3075042492329361</v>
       </c>
       <c r="K159" s="151" t="n">
-        <v>0.2668663304445173</v>
+        <v>0.2721899596042816</v>
       </c>
       <c r="L159" s="151" t="n">
-        <v>0.1514180498478056</v>
+        <v>0.1569705909572128</v>
       </c>
       <c r="M159" s="151" t="n">
-        <v>0.304136451395162</v>
+        <v>0.3074746951909192</v>
       </c>
       <c r="N159" s="151" t="n">
-        <v>0.2668367486516327</v>
+        <v>0.2721603778114374</v>
       </c>
       <c r="O159" s="151" t="n">
-        <v>0.1514243703338647</v>
+        <v>0.1569769114431724</v>
       </c>
       <c r="P159" s="151" t="n">
-        <v>0.3041427844042148</v>
+        <v>0.307481028199953</v>
       </c>
       <c r="Q159" s="151" t="n">
-        <v>0.2668430876072663</v>
+        <v>0.2721667167670597</v>
       </c>
       <c r="R159" s="150" t="n">
-        <v>0.1349810410827771</v>
+        <v>0.1368913591210255</v>
       </c>
       <c r="S159" s="150" t="n">
-        <v>0.1349621965953671</v>
+        <v>0.1368725146336156</v>
       </c>
       <c r="T159" s="151" t="n">
-        <v>0.1440228049458968</v>
+        <v>0.1477172220764529</v>
       </c>
       <c r="U159" s="151" t="n">
-        <v>0.299705284602134</v>
+        <v>0.3019264054948317</v>
       </c>
       <c r="V159" s="151" t="n">
-        <v>0.259748028548601</v>
+        <v>0.2632901377160011</v>
       </c>
       <c r="W159" s="151" t="n">
-        <v>0.1440031798674944</v>
+        <v>0.1476975969983202</v>
       </c>
       <c r="X159" s="151" t="n">
-        <v>0.2996856206397765</v>
+        <v>0.3019067415325195</v>
       </c>
       <c r="Y159" s="151" t="n">
-        <v>0.2597283461220796</v>
+        <v>0.2632704552895065</v>
       </c>
       <c r="Z159" s="151" t="n">
-        <v>0.1440073852414866</v>
+        <v>0.1477018023722461</v>
       </c>
       <c r="AA159" s="151" t="n">
-        <v>0.299689834346019</v>
+        <v>0.3019109552387494</v>
       </c>
       <c r="AB159" s="151" t="n">
-        <v>0.2597325637849158</v>
+        <v>0.2632746729523353</v>
       </c>
     </row>
     <row r="160" ht="15" customHeight="1">
@@ -17707,70 +17707,70 @@
       </c>
       <c r="F160" s="123" t="inlineStr"/>
       <c r="G160" s="152" t="n">
-        <v>0.4530573527276018</v>
+        <v>0.4560956881600446</v>
       </c>
       <c r="H160" s="152" t="n">
-        <v>0.3791642058908935</v>
+        <v>0.3822025413233363</v>
       </c>
       <c r="I160" s="153" t="n">
-        <v>0.3922828118807444</v>
+        <v>0.3978353529897461</v>
       </c>
       <c r="J160" s="153" t="n">
-        <v>0.4534803573460149</v>
+        <v>0.4568186011417041</v>
       </c>
       <c r="K160" s="153" t="n">
-        <v>0.5567118370909494</v>
+        <v>0.5620354662507137</v>
       </c>
       <c r="L160" s="153" t="n">
-        <v>0.3922533162794773</v>
+        <v>0.3978058573888845</v>
       </c>
       <c r="M160" s="153" t="n">
-        <v>0.4534508033039301</v>
+        <v>0.4567890470996873</v>
       </c>
       <c r="N160" s="153" t="n">
-        <v>0.5566822552980648</v>
+        <v>0.5620058844578695</v>
       </c>
       <c r="O160" s="153" t="n">
-        <v>0.3922596367655365</v>
+        <v>0.3978121778748441</v>
       </c>
       <c r="P160" s="153" t="n">
-        <v>0.4534571363129829</v>
+        <v>0.456795380108721</v>
       </c>
       <c r="Q160" s="153" t="n">
-        <v>0.5566885942536983</v>
+        <v>0.5620122234134919</v>
       </c>
       <c r="R160" s="152" t="n">
-        <v>0.2864034116341725</v>
+        <v>0.2883137296724209</v>
       </c>
       <c r="S160" s="152" t="n">
-        <v>0.2863845671467626</v>
+        <v>0.2882948851850111</v>
       </c>
       <c r="T160" s="153" t="n">
-        <v>0.3042640200005229</v>
+        <v>0.3079584371310791</v>
       </c>
       <c r="U160" s="153" t="n">
-        <v>0.3990525003544551</v>
+        <v>0.4012736212471528</v>
       </c>
       <c r="V160" s="153" t="n">
-        <v>0.4525985061854596</v>
+        <v>0.4561406153528597</v>
       </c>
       <c r="W160" s="153" t="n">
-        <v>0.3042443949221205</v>
+        <v>0.3079388120529464</v>
       </c>
       <c r="X160" s="153" t="n">
-        <v>0.3990328363920976</v>
+        <v>0.4012539572848405</v>
       </c>
       <c r="Y160" s="153" t="n">
-        <v>0.4525788237589382</v>
+        <v>0.4561209329263651</v>
       </c>
       <c r="Z160" s="153" t="n">
-        <v>0.3042486002961127</v>
+        <v>0.3079430174268722</v>
       </c>
       <c r="AA160" s="153" t="n">
-        <v>0.3990370500983401</v>
+        <v>0.4012581709910705</v>
       </c>
       <c r="AB160" s="153" t="n">
-        <v>0.4525830414217744</v>
+        <v>0.4561251505891939</v>
       </c>
     </row>
     <row r="161" ht="15" customHeight="1">
@@ -17801,70 +17801,70 @@
       </c>
       <c r="F161" s="123" t="inlineStr"/>
       <c r="G161" s="152" t="n">
-        <v>1.71709536116388</v>
+        <v>2.12354528738614</v>
       </c>
       <c r="H161" s="152" t="n">
-        <v>1.63932447237903</v>
+        <v>2.045774398601298</v>
       </c>
       <c r="I161" s="153" t="n">
-        <v>3.840973312069803</v>
+        <v>4.696214229179318</v>
       </c>
       <c r="J161" s="153" t="n">
-        <v>2.437790821299018</v>
+        <v>2.923807338058453</v>
       </c>
       <c r="K161" s="153" t="n">
-        <v>3.67523902935652</v>
+        <v>4.445550738342776</v>
       </c>
       <c r="L161" s="153" t="n">
-        <v>3.84091807921999</v>
+        <v>4.696158996035751</v>
       </c>
       <c r="M161" s="153" t="n">
-        <v>2.437737965759786</v>
+        <v>2.923754482170276</v>
       </c>
       <c r="N161" s="153" t="n">
-        <v>3.675187653863974</v>
+        <v>4.44549936268872</v>
       </c>
       <c r="O161" s="153" t="n">
-        <v>3.840929914725353</v>
+        <v>4.696170831625423</v>
       </c>
       <c r="P161" s="153" t="n">
-        <v>2.437749291834332</v>
+        <v>2.923765808342443</v>
       </c>
       <c r="Q161" s="153" t="n">
-        <v>3.675198662845537</v>
+        <v>4.44551037171547</v>
       </c>
       <c r="R161" s="152" t="n">
-        <v>1.09260513458614</v>
+        <v>1.348155794798428</v>
       </c>
       <c r="S161" s="152" t="n">
-        <v>1.09257346731619</v>
+        <v>1.348124127528474</v>
       </c>
       <c r="T161" s="153" t="n">
-        <v>2.611380326955709</v>
+        <v>3.180420093234884</v>
       </c>
       <c r="U161" s="153" t="n">
-        <v>1.734658316379735</v>
+        <v>2.058032373410724</v>
       </c>
       <c r="V161" s="153" t="n">
-        <v>2.542071709751747</v>
+        <v>3.054603308830421</v>
       </c>
       <c r="W161" s="153" t="n">
-        <v>2.611343577441835</v>
+        <v>3.18038334352556</v>
       </c>
       <c r="X161" s="153" t="n">
-        <v>1.734623148623972</v>
+        <v>2.057997205422789</v>
       </c>
       <c r="Y161" s="153" t="n">
-        <v>2.542037526754084</v>
+        <v>3.054569125725295</v>
       </c>
       <c r="Z161" s="153" t="n">
-        <v>2.611351452267597</v>
+        <v>3.180391218407416</v>
       </c>
       <c r="AA161" s="153" t="n">
-        <v>1.734630684496829</v>
+        <v>2.058004741360597</v>
       </c>
       <c r="AB161" s="153" t="n">
-        <v>2.542044851647188</v>
+        <v>3.054576450648465</v>
       </c>
     </row>
     <row r="162" ht="15" customHeight="1">
@@ -18092,7 +18092,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -18375,7 +18374,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
@@ -19445,12 +19443,12 @@
     <row r="17">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>New-build capital cost (working assumption, 20 Oct 2026): CCGT US$1,200/kW, gas engine US$1,100/kW, OCGT US$700/kW</t>
+          <t>Capital cost (working assumption, 20 Oct 2026, market +25%): existing CCGT US$600/kW; new CCGT US$1,500/kW, gas engine US$1,375/kW, OCGT US$875/kW</t>
         </is>
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>Market-level working values chosen 20 Oct 2026 in response to Wärtsilä and Quezon Power comments (GAIR matrix rows 119, 412); to be sourced in the Reference Parameters Resolution</t>
+          <t>Market-level working values raised 20 Oct 2026 (+25%, EPC and turbine cost inflation), in response to Wärtsilä and Quezon Power comments (GAIR matrix rows 119, 412); to be sourced in the Reference Parameters Resolution</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Fuel what-if from URR bills (Jul/Aug 2026 supply) in decks and models
Rates deck: new what-if slides (draft GATP + billed fuel commodity +
CLLC certified at min(billed, cap)) against MERALCO actuals for the same
supply month; JKM all-in made VAT-exclusive; no previous-draft or +25%
references in either deck. Models: GATP Build-up what-if block replaces
the previous-draft block. FinModel_Summary: new Fuel_WhatIf sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6VUATAmWPQdQ6XxJGJU7F
</commit_message>
<xml_diff>
--- a/FinModel_Summary.xlsx
+++ b/FinModel_Summary.xlsx
@@ -11,14 +11,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GATP_Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GATP_Composition" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rates" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOR_Conditions" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical_CF" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuel_WhatIf" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOR_Conditions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical_CF" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Parameters'!$A$9:$AB$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Parameters'!$A$9:$AB$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -35,7 +36,7 @@
     <numFmt numFmtId="169" formatCode="0.00000"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
-  <fonts count="51">
+  <fonts count="57">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -279,8 +280,41 @@
       <color rgb="001E7B4F"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="0052606D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="0052606D"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="26">
+  <fills count="32">
     <fill>
       <patternFill/>
     </fill>
@@ -422,8 +456,38 @@
         <bgColor rgb="00DCE6F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F8A8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006C3FA0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F0FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D3EEEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E9E1F4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -506,11 +570,25 @@
         <color rgb="00C0392B"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9DEE5"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9DEE5"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9DEE5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9DEE5"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="154">
+  <cellXfs count="168">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -858,6 +936,46 @@
     </xf>
     <xf numFmtId="165" fontId="36" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="26" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="27" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="28" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="54" fillId="29" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="29" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="54" fillId="29" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="54" fillId="29" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="54" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="55" fillId="30" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="55" fillId="31" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1798,6 +1916,287 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Reference for every assumption</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="67" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+      <c r="B3" s="67" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C3" s="67" t="inlineStr">
+        <is>
+          <t>File / location</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>Lots, capacity factor bands, delivery year, supply period</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>DOE Terms of Reference (Annex B), Sec. 1.1, 1.2, 4.2, 18.3</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>GAIR RCM/Terms of Reference/Annex B - Terms of Reference.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>30-year cost recovery; zero construction for existing plants</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>ERC basis (plant economic life); instruction of 20 Oct 2026; GAIR Table 1</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>franz_som_working draft_1.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Historical capacity factor (Fin90)</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Meralco Breakdown of Generation Charge, Jan 2024–Sep 2026 (First Gen Santa Rita, San Lorenzo; SPPC Ilijan; EERI)</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>xxxxxxx/*_gc_table.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>Capital cost, fixed and variable O&amp;M, heat rate, construction, unit size</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Draft Resolution 2 values (DOE/EPC 2026 benchmarks, LTSA, cheat sheet)</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>claudenumbers/01_master_numbers_cheat_sheet.md; whisper/scripts/cases.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Lazard comparison (CCGT capex, O&amp;M, heat rate)</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Lazard LCOE v19 (June 2026) as cited in the GAIR workbook</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>mid_merit_gas_rates.xlsx, O&amp;M Rebasing tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>First Gen historical O&amp;M (Santa Rita / San Lorenzo 1996 PPA, re-based May 2026)</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>ERC Case No. 2004-74 PPA rates, CPI re-basing</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>mid_merit_gas_rates.xlsx, O&amp;M Rebasing tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>Existing-plant capital cost US$450/kW; brownfield US$600/kW (San Gabriel, EERI)</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>GAIR workbook / cheat sheet</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>mid_merit_gas_rates.xlsx; cheat sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>Financing: 70:30, Kd 8%, 15-yr tenor, Re 14%</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Draft Resolution 2 (Annex A.9–A.12)</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>cheat sheet; whisper/scripts/engine.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Logistics caps (CLLC)</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Draft Resolution 2 caps; BOG removed per working Rules Sec. 17</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>cases.py; franz_som_working draft_1.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>PhP/US$ 62.756</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>BSP reference rate, 25 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>whisper/scripts/cases.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>Taxes (CIT 25%, VAT 12%, RPT 2%, LBT 1%, WHT, GRT, DST)</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>CREATE Act (RA 11534), NIRC, LGC — model defaults</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>whisper/ERC Mid-Merit Financial Model.xlsm (Sensitivity Analysis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>ER 1-94 PhP 0.03/kWh</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>DOE DC2025-10-0023; GAIR 8.8.3</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>naruto C90</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>Model template</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>naruto.xlsm (blank ERC Mid-Merit Financial Model)</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>GAIR RCM/whisper/naruto.xlsm</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>Capital cost (working assumption, 20 Oct 2026, market +25%): existing CCGT US$600/kW; new CCGT US$1,500/kW, gas engine US$1,375/kW, OCGT US$875/kW</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Market-level working values raised 20 Oct 2026 (+25%, EPC and turbine cost inflation), in response to Wärtsilä and Quezon Power comments (GAIR matrix rows 119, 412); to be sourced in the Reference Parameters Resolution</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>models Fin42/Fin90, cell O34</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4023,6 +4422,7 @@
       <c r="I2" s="69" t="n"/>
       <c r="J2" s="69" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="79" t="inlineStr">
         <is>
@@ -4510,6 +4910,573 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00B45309"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="154" t="inlineStr">
+        <is>
+          <t>What if: draft GATP + fuel actually billed to MERALCO (URR bills, July and August 2026 supply)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="155" t="inlineStr">
+        <is>
+          <t>All PhP/kWh, excl. VAT. CLLC certified = lower of the billed logistics and the cap (Sec. 17, 23). Cap: LNG US$2.20/MMBtu (regas 1.50 + pipeline 0.40 + storage 0.30), Malampaya US$0.40 (pipeline). GATP linked to the Rates sheet. Blue cells are inputs from the bills.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="156" t="inlineStr">
+        <is>
+          <t>Plant – supply month</t>
+        </is>
+      </c>
+      <c r="B4" s="156" t="inlineStr">
+        <is>
+          <t>Fuel mix</t>
+        </is>
+      </c>
+      <c r="C4" s="156" t="inlineStr">
+        <is>
+          <t>LNG share</t>
+        </is>
+      </c>
+      <c r="D4" s="156" t="inlineStr">
+        <is>
+          <t>Malampaya share</t>
+        </is>
+      </c>
+      <c r="E4" s="156" t="inlineStr">
+        <is>
+          <t>Heat rate (Btu/kWh)</t>
+        </is>
+      </c>
+      <c r="F4" s="156" t="inlineStr">
+        <is>
+          <t>Bill FX (PhP/US$)</t>
+        </is>
+      </c>
+      <c r="G4" s="156" t="inlineStr">
+        <is>
+          <t>Billed fuel commodity</t>
+        </is>
+      </c>
+      <c r="H4" s="156" t="inlineStr">
+        <is>
+          <t>Billed logistics</t>
+        </is>
+      </c>
+      <c r="I4" s="156" t="inlineStr">
+        <is>
+          <t>CLLC cap</t>
+        </is>
+      </c>
+      <c r="J4" s="156" t="inlineStr">
+        <is>
+          <t>CLLC certified</t>
+        </is>
+      </c>
+      <c r="K4" s="157" t="inlineStr">
+        <is>
+          <t>GATP Case A</t>
+        </is>
+      </c>
+      <c r="L4" s="158" t="inlineStr">
+        <is>
+          <t>GATP Case B</t>
+        </is>
+      </c>
+      <c r="M4" s="157" t="inlineStr">
+        <is>
+          <t>All-in Case A</t>
+        </is>
+      </c>
+      <c r="N4" s="158" t="inlineStr">
+        <is>
+          <t>All-in Case B</t>
+        </is>
+      </c>
+      <c r="O4" s="156" t="inlineStr">
+        <is>
+          <t>MERALCO actual</t>
+        </is>
+      </c>
+      <c r="P4" s="156" t="inlineStr">
+        <is>
+          <t>Actual minus all-in A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="159" t="inlineStr">
+        <is>
+          <t>Santa Rita – Jul 2026 supply</t>
+        </is>
+      </c>
+      <c r="B5" s="159" t="inlineStr">
+        <is>
+          <t>LNG 58% / Malampaya 27% / liquid 15%</t>
+        </is>
+      </c>
+      <c r="C5" s="160" t="n">
+        <v>0.5815</v>
+      </c>
+      <c r="D5" s="160" t="n">
+        <v>0.2712</v>
+      </c>
+      <c r="E5" s="161" t="n">
+        <v>6350</v>
+      </c>
+      <c r="F5" s="162" t="n">
+        <v>61.945</v>
+      </c>
+      <c r="G5" s="163" t="n">
+        <v>7.7128</v>
+      </c>
+      <c r="H5" s="163" t="n">
+        <v>1.2633</v>
+      </c>
+      <c r="I5" s="164">
+        <f>(C5*2.2+D5*0.4)*E5/1000000*F5</f>
+        <v/>
+      </c>
+      <c r="J5" s="164">
+        <f>MIN(H5,I5)</f>
+        <v/>
+      </c>
+      <c r="K5" s="164">
+        <f>Rates!F5</f>
+        <v/>
+      </c>
+      <c r="L5" s="164">
+        <f>Rates!G5</f>
+        <v/>
+      </c>
+      <c r="M5" s="165">
+        <f>K5+G5+J5</f>
+        <v/>
+      </c>
+      <c r="N5" s="166">
+        <f>L5+G5+J5</f>
+        <v/>
+      </c>
+      <c r="O5" s="163" t="n">
+        <v>10.7708</v>
+      </c>
+      <c r="P5" s="164">
+        <f>O5-M5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="159" t="inlineStr">
+        <is>
+          <t>Santa Rita – Aug 2026 supply</t>
+        </is>
+      </c>
+      <c r="B6" s="159" t="inlineStr">
+        <is>
+          <t>100% Malampaya</t>
+        </is>
+      </c>
+      <c r="C6" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="160" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="161" t="n">
+        <v>6350</v>
+      </c>
+      <c r="F6" s="162" t="n">
+        <v>62</v>
+      </c>
+      <c r="G6" s="163" t="n">
+        <v>6.6064</v>
+      </c>
+      <c r="H6" s="163" t="n">
+        <v>1.0785</v>
+      </c>
+      <c r="I6" s="164">
+        <f>(C6*2.2+D6*0.4)*E6/1000000*F6</f>
+        <v/>
+      </c>
+      <c r="J6" s="164">
+        <f>MIN(H6,I6)</f>
+        <v/>
+      </c>
+      <c r="K6" s="164">
+        <f>Rates!F5</f>
+        <v/>
+      </c>
+      <c r="L6" s="164">
+        <f>Rates!G5</f>
+        <v/>
+      </c>
+      <c r="M6" s="165">
+        <f>K6+G6+J6</f>
+        <v/>
+      </c>
+      <c r="N6" s="166">
+        <f>L6+G6+J6</f>
+        <v/>
+      </c>
+      <c r="O6" s="163" t="n">
+        <v>6.9472</v>
+      </c>
+      <c r="P6" s="164">
+        <f>O6-M6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="159" t="inlineStr">
+        <is>
+          <t>San Lorenzo – Jul 2026 supply</t>
+        </is>
+      </c>
+      <c r="B7" s="159" t="inlineStr">
+        <is>
+          <t>LNG 65% / Malampaya 35%</t>
+        </is>
+      </c>
+      <c r="C7" s="160" t="n">
+        <v>0.6466</v>
+      </c>
+      <c r="D7" s="160" t="n">
+        <v>0.3534</v>
+      </c>
+      <c r="E7" s="161" t="n">
+        <v>6350</v>
+      </c>
+      <c r="F7" s="162" t="n">
+        <v>61.945</v>
+      </c>
+      <c r="G7" s="163" t="n">
+        <v>7.4562</v>
+      </c>
+      <c r="H7" s="163" t="n">
+        <v>1.1113</v>
+      </c>
+      <c r="I7" s="164">
+        <f>(C7*2.2+D7*0.4)*E7/1000000*F7</f>
+        <v/>
+      </c>
+      <c r="J7" s="164">
+        <f>MIN(H7,I7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="164">
+        <f>Rates!F5</f>
+        <v/>
+      </c>
+      <c r="L7" s="164">
+        <f>Rates!G5</f>
+        <v/>
+      </c>
+      <c r="M7" s="165">
+        <f>K7+G7+J7</f>
+        <v/>
+      </c>
+      <c r="N7" s="166">
+        <f>L7+G7+J7</f>
+        <v/>
+      </c>
+      <c r="O7" s="163" t="n">
+        <v>10.6771</v>
+      </c>
+      <c r="P7" s="164">
+        <f>O7-M7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="159" t="inlineStr">
+        <is>
+          <t>San Lorenzo – Aug 2026 supply</t>
+        </is>
+      </c>
+      <c r="B8" s="159" t="inlineStr">
+        <is>
+          <t>100% Malampaya</t>
+        </is>
+      </c>
+      <c r="C8" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="160" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="161" t="n">
+        <v>6350</v>
+      </c>
+      <c r="F8" s="162" t="n">
+        <v>62.498</v>
+      </c>
+      <c r="G8" s="163" t="n">
+        <v>6.4776</v>
+      </c>
+      <c r="H8" s="163" t="n">
+        <v>1.0884</v>
+      </c>
+      <c r="I8" s="164">
+        <f>(C8*2.2+D8*0.4)*E8/1000000*F8</f>
+        <v/>
+      </c>
+      <c r="J8" s="164">
+        <f>MIN(H8,I8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="164">
+        <f>Rates!F5</f>
+        <v/>
+      </c>
+      <c r="L8" s="164">
+        <f>Rates!G5</f>
+        <v/>
+      </c>
+      <c r="M8" s="165">
+        <f>K8+G8+J8</f>
+        <v/>
+      </c>
+      <c r="N8" s="166">
+        <f>L8+G8+J8</f>
+        <v/>
+      </c>
+      <c r="O8" s="163" t="n">
+        <v>9.814399999999999</v>
+      </c>
+      <c r="P8" s="164">
+        <f>O8-M8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="159" t="inlineStr">
+        <is>
+          <t>Ilijan (2024 PSA) – Jul 2026 supply</t>
+        </is>
+      </c>
+      <c r="B9" s="159" t="inlineStr">
+        <is>
+          <t>100% LNG (Brent-linked)</t>
+        </is>
+      </c>
+      <c r="C9" s="160" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="161" t="n">
+        <v>6350</v>
+      </c>
+      <c r="F9" s="162" t="n">
+        <v>61.847</v>
+      </c>
+      <c r="G9" s="163" t="n">
+        <v>9.636100000000001</v>
+      </c>
+      <c r="H9" s="163" t="n">
+        <v>0.5239</v>
+      </c>
+      <c r="I9" s="164">
+        <f>(C9*2.2+D9*0.4)*E9/1000000*F9</f>
+        <v/>
+      </c>
+      <c r="J9" s="164">
+        <f>MIN(H9,I9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="164">
+        <f>Rates!F6</f>
+        <v/>
+      </c>
+      <c r="L9" s="164">
+        <f>Rates!G6</f>
+        <v/>
+      </c>
+      <c r="M9" s="165">
+        <f>K9+G9+J9</f>
+        <v/>
+      </c>
+      <c r="N9" s="166">
+        <f>L9+G9+J9</f>
+        <v/>
+      </c>
+      <c r="O9" s="163" t="n">
+        <v>13.0017</v>
+      </c>
+      <c r="P9" s="164">
+        <f>O9-M9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="159" t="inlineStr">
+        <is>
+          <t>Ilijan (2024 PSA) – Aug 2026 supply</t>
+        </is>
+      </c>
+      <c r="B10" s="159" t="inlineStr">
+        <is>
+          <t>100% LNG (Brent-linked)</t>
+        </is>
+      </c>
+      <c r="C10" s="160" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="161" t="n">
+        <v>6350</v>
+      </c>
+      <c r="F10" s="162" t="n">
+        <v>61.738</v>
+      </c>
+      <c r="G10" s="163" t="n">
+        <v>10.2713</v>
+      </c>
+      <c r="H10" s="163" t="n">
+        <v>0.5256999999999999</v>
+      </c>
+      <c r="I10" s="164">
+        <f>(C10*2.2+D10*0.4)*E10/1000000*F10</f>
+        <v/>
+      </c>
+      <c r="J10" s="164">
+        <f>MIN(H10,I10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="164">
+        <f>Rates!F6</f>
+        <v/>
+      </c>
+      <c r="L10" s="164">
+        <f>Rates!G6</f>
+        <v/>
+      </c>
+      <c r="M10" s="165">
+        <f>K10+G10+J10</f>
+        <v/>
+      </c>
+      <c r="N10" s="166">
+        <f>L10+G10+J10</f>
+        <v/>
+      </c>
+      <c r="O10" s="163" t="n">
+        <v>15.4438</v>
+      </c>
+      <c r="P10" s="164">
+        <f>O10-M10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="159" t="inlineStr">
+        <is>
+          <t>EERI Batangas – Aug 2026 supply</t>
+        </is>
+      </c>
+      <c r="B11" s="159" t="inlineStr">
+        <is>
+          <t>100% LNG (Brent-linked</t>
+        </is>
+      </c>
+      <c r="C11" s="160" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="161" t="n">
+        <v>6100</v>
+      </c>
+      <c r="F11" s="162" t="n">
+        <v>61.8507</v>
+      </c>
+      <c r="G11" s="163" t="n">
+        <v>8.849</v>
+      </c>
+      <c r="H11" s="163" t="n">
+        <v>0.453</v>
+      </c>
+      <c r="I11" s="164">
+        <f>(C11*2.2+D11*0.4)*E11/1000000*F11</f>
+        <v/>
+      </c>
+      <c r="J11" s="164">
+        <f>MIN(H11,I11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="164">
+        <f>Rates!F7</f>
+        <v/>
+      </c>
+      <c r="L11" s="164">
+        <f>Rates!G7</f>
+        <v/>
+      </c>
+      <c r="M11" s="165">
+        <f>K11+G11+J11</f>
+        <v/>
+      </c>
+      <c r="N11" s="166">
+        <f>L11+G11+J11</f>
+        <v/>
+      </c>
+      <c r="O11" s="163" t="n">
+        <v>15.8623</v>
+      </c>
+      <c r="P11" s="164">
+        <f>O11-M11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="167" t="inlineStr">
+        <is>
+          <t>Sources: MERALCO URR power-supply bills in URRnew/ (Santa Rita PB-41000020/21; San Lorenzo PB-41000019/20; SPPC 211 MECO 2607/2608 Final; EERI 802 EERI 2608 Final). MERALCO actual = Breakdown of Generation Charge for the following billing month (Aug and Sep 2026). No September supply-month bills were available. Ilijan and EERI fuel commodity includes ocean freight (delivered LNG); their logistics are the PHLNG terminal fee and PhP import costs.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A13:P13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4659,7 +5626,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18065,7 +19032,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18397,7 +19364,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19179,285 +20146,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="55" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="18" t="inlineStr">
-        <is>
-          <t>Reference for every assumption</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="67" t="inlineStr">
-        <is>
-          <t>Assumption</t>
-        </is>
-      </c>
-      <c r="B3" s="67" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="C3" s="67" t="inlineStr">
-        <is>
-          <t>File / location</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>Lots, capacity factor bands, delivery year, supply period</t>
-        </is>
-      </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>DOE Terms of Reference (Annex B), Sec. 1.1, 1.2, 4.2, 18.3</t>
-        </is>
-      </c>
-      <c r="C4" s="19" t="inlineStr">
-        <is>
-          <t>GAIR RCM/Terms of Reference/Annex B - Terms of Reference.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>30-year cost recovery; zero construction for existing plants</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>ERC basis (plant economic life); instruction of 20 Oct 2026; GAIR Table 1</t>
-        </is>
-      </c>
-      <c r="C5" s="19" t="inlineStr">
-        <is>
-          <t>franz_som_working draft_1.docx</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>Historical capacity factor (Fin90)</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Meralco Breakdown of Generation Charge, Jan 2024–Sep 2026 (First Gen Santa Rita, San Lorenzo; SPPC Ilijan; EERI)</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>xxxxxxx/*_gc_table.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>Capital cost, fixed and variable O&amp;M, heat rate, construction, unit size</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>Draft Resolution 2 values (DOE/EPC 2026 benchmarks, LTSA, cheat sheet)</t>
-        </is>
-      </c>
-      <c r="C7" s="19" t="inlineStr">
-        <is>
-          <t>claudenumbers/01_master_numbers_cheat_sheet.md; whisper/scripts/cases.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>Lazard comparison (CCGT capex, O&amp;M, heat rate)</t>
-        </is>
-      </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>Lazard LCOE v19 (June 2026) as cited in the GAIR workbook</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>mid_merit_gas_rates.xlsx, O&amp;M Rebasing tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>First Gen historical O&amp;M (Santa Rita / San Lorenzo 1996 PPA, re-based May 2026)</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>ERC Case No. 2004-74 PPA rates, CPI re-basing</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="inlineStr">
-        <is>
-          <t>mid_merit_gas_rates.xlsx, O&amp;M Rebasing tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>Existing-plant capital cost US$450/kW; brownfield US$600/kW (San Gabriel, EERI)</t>
-        </is>
-      </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>GAIR workbook / cheat sheet</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>mid_merit_gas_rates.xlsx; cheat sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>Financing: 70:30, Kd 8%, 15-yr tenor, Re 14%</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>Draft Resolution 2 (Annex A.9–A.12)</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="inlineStr">
-        <is>
-          <t>cheat sheet; whisper/scripts/engine.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>Logistics caps (CLLC)</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>Draft Resolution 2 caps; BOG removed per working Rules Sec. 17</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>cases.py; franz_som_working draft_1.docx</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>PhP/US$ 62.756</t>
-        </is>
-      </c>
-      <c r="B13" s="19" t="inlineStr">
-        <is>
-          <t>BSP reference rate, 25 Sep 2026</t>
-        </is>
-      </c>
-      <c r="C13" s="19" t="inlineStr">
-        <is>
-          <t>whisper/scripts/cases.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>Taxes (CIT 25%, VAT 12%, RPT 2%, LBT 1%, WHT, GRT, DST)</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>CREATE Act (RA 11534), NIRC, LGC — model defaults</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>whisper/ERC Mid-Merit Financial Model.xlsm (Sensitivity Analysis)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>ER 1-94 PhP 0.03/kWh</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>DOE DC2025-10-0023; GAIR 8.8.3</t>
-        </is>
-      </c>
-      <c r="C15" s="19" t="inlineStr">
-        <is>
-          <t>naruto C90</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>Model template</t>
-        </is>
-      </c>
-      <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>naruto.xlsm (blank ERC Mid-Merit Financial Model)</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="inlineStr">
-        <is>
-          <t>GAIR RCM/whisper/naruto.xlsm</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>Capital cost (working assumption, 20 Oct 2026, market +25%): existing CCGT US$600/kW; new CCGT US$1,500/kW, gas engine US$1,375/kW, OCGT US$875/kW</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="inlineStr">
-        <is>
-          <t>Market-level working values raised 20 Oct 2026 (+25%, EPC and turbine cost inflation), in response to Wärtsilä and Quezon Power comments (GAIR matrix rows 119, 412); to be sourced in the Reference Parameters Resolution</t>
-        </is>
-      </c>
-      <c r="C17" s="19" t="inlineStr">
-        <is>
-          <t>models Fin42/Fin90, cell O34</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>